<commit_message>
Admin tools: add products, free Featured, Featured rate list, ad rates and ads, reports
- Products: + Add product (RGBKart Official or any seller, live at once); Make Featured (free)
- Featured & ads: rate list by duration (7/15/30 days); ad price per day for three ad spaces;
  create ads (own or for a seller) shown on the home page and category sidebar
- Reports: daily/weekly/monthly/yearly/custom with visitors, sign-ups, listings, income,
  charts and CSV download; visitor counting on shop pages (random device id, no IP)
- Sell an item: one-time sellers choose a Featured duration
Database: 0018_admin_tools.sql

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="235">
   <si>
     <t xml:space="preserve">RGBKart Marketplace – Project Plan</t>
   </si>
@@ -531,7 +531,7 @@
     <t xml:space="preserve">Admin sets packages: placement (home, category top), rate (৳) and duration (days)</t>
   </si>
   <si>
-    <t xml:space="preserve">Built 22 Oct (featured_plans.sql): admin sets plans (default ৳50 / 30 days + benefits); sellers and one-time sellers choose Free or Featured. Admin starts Featured after payment; it ends by itself (contact_messages.sql)</t>
+    <t xml:space="preserve">Rate list (7/15/30 days, admin-editable); sellers pick a duration; admin can give Featured free (Products → Make Featured free). 0018_admin_tools.sql</t>
   </si>
   <si>
     <t xml:space="preserve">5.5</t>
@@ -543,7 +543,7 @@
     <t xml:space="preserve">Admin defines ad types (home banner, category banner, sidebar, popup), size, rate and duration</t>
   </si>
   <si>
-    <t xml:space="preserve">Rates editable any time; already-paid ads keep their price</t>
+    <t xml:space="preserve">23 Oct: Admin → Featured &amp; ads: price per day for Home banner strip, Home mid-page banner, Category sidebar; admin creates ads (own or for a seller), shown on the site</t>
   </si>
   <si>
     <t xml:space="preserve">5.6</t>
@@ -576,6 +576,9 @@
     <t xml:space="preserve">Featured items and ads switch on at approval, switch off at end date; reminder before expiry</t>
   </si>
   <si>
+    <t xml:space="preserve">Featured and ads end by themselves on their end date. Reminders before expiry still to do</t>
+  </si>
+  <si>
     <t xml:space="preserve">5.9</t>
   </si>
   <si>
@@ -595,6 +598,9 @@
   </si>
   <si>
     <t xml:space="preserve">Sales, orders, featured &amp; ad income, top sellers; export</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 Oct: Admin → Reports: daily/weekly/monthly/yearly/custom; visitors, sign-ups, listings, Featured &amp; ad income; charts; CSV download. Sales/orders come with checkout</t>
   </si>
   <si>
     <t xml:space="preserve">5.11</t>
@@ -2551,7 +2557,7 @@
       </c>
       <c r="J42" s="10"/>
     </row>
-    <row r="43" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="n">
         <v>5</v>
       </c>
@@ -2582,7 +2588,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="11" t="n">
         <v>5</v>
       </c>
@@ -2599,9 +2605,11 @@
         <v>164</v>
       </c>
       <c r="F44" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="G44" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G44" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H44" s="8"/>
       <c r="I44" s="14" t="str">
         <f aca="false">IF(AND(G44&lt;&gt;"",H44&lt;&gt;""),H44-G44+1,"")</f>
@@ -2686,15 +2694,19 @@
         <v>175</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="G47" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G47" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H47" s="8"/>
       <c r="I47" s="14" t="str">
         <f aca="false">IF(AND(G47&lt;&gt;"",H47&lt;&gt;""),H47-G47+1,"")</f>
         <v/>
       </c>
-      <c r="J47" s="10"/>
+      <c r="J47" s="10" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="11" t="n">
@@ -2704,13 +2716,13 @@
         <v>148</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D48" s="12" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E48" s="12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F48" s="7" t="s">
         <v>28</v>
@@ -2724,10 +2736,10 @@
         <v/>
       </c>
       <c r="J48" s="10" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="n">
         <v>5</v>
       </c>
@@ -2735,24 +2747,28 @@
         <v>148</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D49" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E49" s="12" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="G49" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G49" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H49" s="8"/>
       <c r="I49" s="14" t="str">
         <f aca="false">IF(AND(G49&lt;&gt;"",H49&lt;&gt;""),H49-G49+1,"")</f>
         <v/>
       </c>
-      <c r="J49" s="10"/>
+      <c r="J49" s="10" t="s">
+        <v>184</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="n">
@@ -2762,13 +2778,13 @@
         <v>148</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F50" s="7" t="s">
         <v>99</v>
@@ -2786,16 +2802,16 @@
         <v>6</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F51" s="7" t="s">
         <v>99</v>
@@ -2813,16 +2829,16 @@
         <v>6</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F52" s="7" t="s">
         <v>99</v>
@@ -2840,16 +2856,16 @@
         <v>6</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F53" s="7" t="s">
         <v>99</v>
@@ -2867,16 +2883,16 @@
         <v>6</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F54" s="7" t="s">
         <v>99</v>
@@ -2894,16 +2910,16 @@
         <v>6</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F55" s="7" t="s">
         <v>99</v>
@@ -2921,16 +2937,16 @@
         <v>7</v>
       </c>
       <c r="B56" s="12" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D56" s="12" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E56" s="12" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="F56" s="7" t="s">
         <v>99</v>
@@ -2948,16 +2964,16 @@
         <v>7</v>
       </c>
       <c r="B57" s="12" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F57" s="7" t="s">
         <v>99</v>
@@ -2969,7 +2985,7 @@
         <v/>
       </c>
       <c r="J57" s="10" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2977,16 +2993,16 @@
         <v>7</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D58" s="12" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="E58" s="12" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="F58" s="7" t="s">
         <v>99</v>
@@ -3004,16 +3020,16 @@
         <v>7</v>
       </c>
       <c r="B59" s="12" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E59" s="12" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F59" s="7" t="s">
         <v>99</v>
@@ -3031,16 +3047,16 @@
         <v>7</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D60" s="12" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="E60" s="12" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F60" s="7" t="s">
         <v>99</v>
@@ -3058,16 +3074,16 @@
         <v>7</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C61" s="13" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="E61" s="12" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F61" s="7" t="s">
         <v>99</v>
@@ -3085,16 +3101,16 @@
         <v>7</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D62" s="12" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E62" s="12" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F62" s="7" t="s">
         <v>99</v>
@@ -3165,7 +3181,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3176,7 +3192,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>16</v>
@@ -3185,19 +3201,19 @@
         <v>28</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>99</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3417,7 +3433,7 @@
       </c>
       <c r="E9" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A9,Plan!$F$5:$F$262,"In progress")</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F9" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A9,Plan!$F$5:$F$262,"Blocked")</f>
@@ -3425,7 +3441,7 @@
       </c>
       <c r="G9" s="15" t="n">
         <f aca="false">C9-D9-E9-F9</f>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H9" s="16" t="n">
         <f aca="false">IF(C9=0,0,D9/C9)</f>
@@ -3445,7 +3461,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C10" s="15" t="n">
         <f aca="false">COUNTIF(Plan!$A$5:$A$262,A10)</f>
@@ -3485,7 +3501,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C11" s="15" t="n">
         <f aca="false">COUNTIF(Plan!$A$5:$A$262,A11)</f>
@@ -3523,7 +3539,7 @@
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18"/>
       <c r="B12" s="18" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C12" s="18" t="n">
         <f aca="false">SUM(C4:C11)</f>
@@ -3535,7 +3551,7 @@
       </c>
       <c r="E12" s="18" t="n">
         <f aca="false">SUM(E4:E11)</f>
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F12" s="18" t="n">
         <f aca="false">SUM(F4:F11)</f>
@@ -3543,7 +3559,7 @@
       </c>
       <c r="G12" s="18" t="n">
         <f aca="false">SUM(G4:G11)</f>
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H12" s="19" t="n">
         <f aca="false">IF(C12=0,0,D12/C12)</f>
@@ -3554,7 +3570,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -3567,7 +3583,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{658E3AE3-70A5-4F28-A698-A8A94C94A433}</x14:id>
+          <x14:id>{1A6C5287-C1C4-4CB7-AF1B-C8DC208DE3FA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3583,7 +3599,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{658E3AE3-70A5-4F28-A698-A8A94C94A433}">
+          <x14:cfRule type="dataBar" id="{1A6C5287-C1C4-4CB7-AF1B-C8DC208DE3FA}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
Seller payments by bKash/Nagad/Upay/Rocket with TrxID; admin Payments queue; seller ad booking
- Sellers pay Featured fees (Sell page, Seller Center) and book + pay for ads (Seller Center → Advertise)
- Admin → Payments: account numbers per method; verify (starts Featured / ad) or reject with reason
- A Transaction ID can be used only once (capitals/spaces ignored)
Database: 0019_payments.sql. Shared form: pay.js

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="236">
   <si>
     <t xml:space="preserve">RGBKart Marketplace – Project Plan</t>
   </si>
@@ -555,6 +555,9 @@
     <t xml:space="preserve">Seller picks a package, uploads banner (ads), pays, sees status and expiry</t>
   </si>
   <si>
+    <t xml:space="preserve">23 Oct: sellers pay Featured fees (Sell page, Seller Center) and book + pay for ads (Seller Center → Advertise). Ad pictures optional</t>
+  </si>
+  <si>
     <t xml:space="preserve">5.7</t>
   </si>
   <si>
@@ -564,7 +567,7 @@
     <t xml:space="preserve">Admin queue for manual payments (bKash, Nagad, bank): check TrxID &amp; amount, approve or reject with reason</t>
   </si>
   <si>
-    <t xml:space="preserve">22 Oct: simple version: admin presses 'Payment received: start' in Featured &amp; ads. TrxID entry by seller still to do; used for order payments too</t>
+    <t xml:space="preserve">23 Oct: Admin → Payments: bKash/Nagad/Upay/Rocket numbers; queue with Verify &amp; start / Reject with reason; each TrxID usable only once (0019_payments.sql). Order payments come with checkout</t>
   </si>
   <si>
     <t xml:space="preserve">5.8</t>
@@ -2619,7 +2622,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="n">
         <v>5</v>
       </c>
@@ -2636,17 +2639,21 @@
         <v>168</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="G45" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G45" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H45" s="8"/>
       <c r="I45" s="14" t="str">
         <f aca="false">IF(AND(G45&lt;&gt;"",H45&lt;&gt;""),H45-G45+1,"")</f>
         <v/>
       </c>
-      <c r="J45" s="10"/>
-    </row>
-    <row r="46" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J45" s="10" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="11" t="n">
         <v>5</v>
       </c>
@@ -2654,13 +2661,13 @@
         <v>148</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D46" s="12" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E46" s="12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F46" s="7" t="s">
         <v>28</v>
@@ -2674,7 +2681,7 @@
         <v/>
       </c>
       <c r="J46" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2685,13 +2692,13 @@
         <v>148</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E47" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F47" s="7" t="s">
         <v>28</v>
@@ -2705,7 +2712,7 @@
         <v/>
       </c>
       <c r="J47" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2716,13 +2723,13 @@
         <v>148</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D48" s="12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E48" s="12" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F48" s="7" t="s">
         <v>28</v>
@@ -2736,7 +2743,7 @@
         <v/>
       </c>
       <c r="J48" s="10" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2747,13 +2754,13 @@
         <v>148</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D49" s="12" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E49" s="12" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F49" s="7" t="s">
         <v>28</v>
@@ -2767,7 +2774,7 @@
         <v/>
       </c>
       <c r="J49" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2778,13 +2785,13 @@
         <v>148</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F50" s="7" t="s">
         <v>99</v>
@@ -2802,16 +2809,16 @@
         <v>6</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F51" s="7" t="s">
         <v>99</v>
@@ -2829,16 +2836,16 @@
         <v>6</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F52" s="7" t="s">
         <v>99</v>
@@ -2856,16 +2863,16 @@
         <v>6</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F53" s="7" t="s">
         <v>99</v>
@@ -2883,16 +2890,16 @@
         <v>6</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F54" s="7" t="s">
         <v>99</v>
@@ -2910,16 +2917,16 @@
         <v>6</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F55" s="7" t="s">
         <v>99</v>
@@ -2937,16 +2944,16 @@
         <v>7</v>
       </c>
       <c r="B56" s="12" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D56" s="12" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E56" s="12" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F56" s="7" t="s">
         <v>99</v>
@@ -2964,16 +2971,16 @@
         <v>7</v>
       </c>
       <c r="B57" s="12" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F57" s="7" t="s">
         <v>99</v>
@@ -2985,7 +2992,7 @@
         <v/>
       </c>
       <c r="J57" s="10" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2993,16 +3000,16 @@
         <v>7</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D58" s="12" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E58" s="12" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F58" s="7" t="s">
         <v>99</v>
@@ -3020,16 +3027,16 @@
         <v>7</v>
       </c>
       <c r="B59" s="12" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E59" s="12" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F59" s="7" t="s">
         <v>99</v>
@@ -3047,16 +3054,16 @@
         <v>7</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D60" s="12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E60" s="12" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F60" s="7" t="s">
         <v>99</v>
@@ -3074,16 +3081,16 @@
         <v>7</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C61" s="13" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E61" s="12" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F61" s="7" t="s">
         <v>99</v>
@@ -3101,16 +3108,16 @@
         <v>7</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D62" s="12" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E62" s="12" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F62" s="7" t="s">
         <v>99</v>
@@ -3181,7 +3188,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3192,7 +3199,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>16</v>
@@ -3201,19 +3208,19 @@
         <v>28</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>99</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3433,7 +3440,7 @@
       </c>
       <c r="E9" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A9,Plan!$F$5:$F$262,"In progress")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F9" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A9,Plan!$F$5:$F$262,"Blocked")</f>
@@ -3441,7 +3448,7 @@
       </c>
       <c r="G9" s="15" t="n">
         <f aca="false">C9-D9-E9-F9</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H9" s="16" t="n">
         <f aca="false">IF(C9=0,0,D9/C9)</f>
@@ -3461,7 +3468,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C10" s="15" t="n">
         <f aca="false">COUNTIF(Plan!$A$5:$A$262,A10)</f>
@@ -3501,7 +3508,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C11" s="15" t="n">
         <f aca="false">COUNTIF(Plan!$A$5:$A$262,A11)</f>
@@ -3539,7 +3546,7 @@
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18"/>
       <c r="B12" s="18" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C12" s="18" t="n">
         <f aca="false">SUM(C4:C11)</f>
@@ -3551,7 +3558,7 @@
       </c>
       <c r="E12" s="18" t="n">
         <f aca="false">SUM(E4:E11)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F12" s="18" t="n">
         <f aca="false">SUM(F4:F11)</f>
@@ -3559,7 +3566,7 @@
       </c>
       <c r="G12" s="18" t="n">
         <f aca="false">SUM(G4:G11)</f>
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H12" s="19" t="n">
         <f aca="false">IF(C12=0,0,D12/C12)</f>
@@ -3570,7 +3577,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -3583,7 +3590,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1A6C5287-C1C4-4CB7-AF1B-C8DC208DE3FA}</x14:id>
+          <x14:id>{57AB1910-F5DB-40D9-BF32-B9C2748016F2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3599,7 +3606,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1A6C5287-C1C4-4CB7-AF1B-C8DC208DE3FA}">
+          <x14:cfRule type="dataBar" id="{57AB1910-F5DB-40D9-BF32-B9C2748016F2}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
Checkout and orders: cart by shop, Cash on Delivery, seller and admin order screens
- cart.html grouped by shop with live prices/stock and delivery choice per shop
- checkout.html: delivery details, Cash on Delivery, one order per shop; guests can order
- orders.html: customers track progress, call/WhatsApp the shop, cancel early
- Seller Center → Orders: confirm, pack, ship (tracking), deliver, cancel; invoice and packing slip; pickup option
- Admin → Orders: all orders, cancel, delivery charges; order figures in Reports
Database: 0020_orders.sql

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="244">
   <si>
     <t xml:space="preserve">RGBKart Marketplace – Project Plan</t>
   </si>
@@ -345,60 +345,72 @@
     <t xml:space="preserve">Add, update, remove items; cart saved to account</t>
   </si>
   <si>
+    <t xml:space="preserve">23 Oct: cart grouped by shop with live prices/stock and delivery choice; saved on the device (moves to the account later)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyer–seller messages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyers message sellers about a product; both reply on the Messages page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Built 22 Oct (messages.html, contact_messages.sql). Only buyer and seller can read a chat. Email/SMS alerts for new messages still to do</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Checkout &amp; Payments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address book</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customers save delivery addresses (division, district, area)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Checkout remembers the last address on the device and fills it from the customer profile; full address book later</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Checkout flow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address → delivery option → payment → review → place order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 Oct: checkout.html, delivery details → Cash on Delivery → one order per shop (0020_orders.sql, place_order checks prices and stock)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash on delivery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COD option with order limits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash on Delivery is the only payment; RGBKart never holds money. Order limits per day in place</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bKash &amp; Nagad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobile wallet payments</t>
+  </si>
+  <si>
     <t xml:space="preserve">Not started</t>
   </si>
   <si>
-    <t xml:space="preserve">2.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buyer–seller messages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buyers message sellers about a product; both reply on the Messages page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Built 22 Oct (messages.html, contact_messages.sql). Only buyer and seller can read a chat. Email/SMS alerts for new messages still to do</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Checkout &amp; Payments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Address book</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customers save delivery addresses (division, district, area)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Checkout flow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Address → delivery option → payment → review → place order</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cash on delivery</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COD option with order limits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bKash &amp; Nagad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mobile wallet payments</t>
-  </si>
-  <si>
     <t xml:space="preserve">Needs merchant accounts</t>
   </si>
   <si>
@@ -444,6 +456,9 @@
     <t xml:space="preserve">One cart with several shops becomes one order per seller</t>
   </si>
   <si>
+    <t xml:space="preserve">One cart with several shops becomes one order per shop (order numbers RGB-YYMMDD-XXXXX)</t>
+  </si>
+  <si>
     <t xml:space="preserve">4.2</t>
   </si>
   <si>
@@ -453,6 +468,9 @@
     <t xml:space="preserve">Sellers accept, pack, mark shipped</t>
   </si>
   <si>
+    <t xml:space="preserve">Seller Center → Orders: confirm, pack, ship (tracking note), deliver, cancel with reason; print invoice and packing slip</t>
+  </si>
+  <si>
     <t xml:space="preserve">4.3</t>
   </si>
   <si>
@@ -474,6 +492,9 @@
     <t xml:space="preserve">Customers see order status and tracking</t>
   </si>
   <si>
+    <t xml:space="preserve">orders.html: customers see progress steps and the shop's delivery info; call/WhatsApp the shop</t>
+  </si>
+  <si>
     <t xml:space="preserve">4.5</t>
   </si>
   <si>
@@ -481,6 +502,9 @@
   </si>
   <si>
     <t xml:space="preserve">Rules for customer and seller cancellations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer cancels while new/confirmed; shop or admin cancels with a reason; stock goes back</t>
   </si>
   <si>
     <t xml:space="preserve">4.6</t>
@@ -2064,7 +2088,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="n">
         <v>2</v>
       </c>
@@ -2081,15 +2105,19 @@
         <v>98</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="G25" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G25" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H25" s="8"/>
       <c r="I25" s="9" t="str">
         <f aca="false">IF(AND(G25&lt;&gt;"",H25&lt;&gt;""),H25-G25+1,"")</f>
         <v/>
       </c>
-      <c r="J25" s="10"/>
+      <c r="J25" s="10" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="n">
@@ -2122,7 +2150,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="n">
         <v>3</v>
       </c>
@@ -2139,17 +2167,21 @@
         <v>107</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="G27" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H27" s="8"/>
       <c r="I27" s="14" t="str">
         <f aca="false">IF(AND(G27&lt;&gt;"",H27&lt;&gt;""),H27-G27+1,"")</f>
         <v/>
       </c>
-      <c r="J27" s="10"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J27" s="10" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="n">
         <v>3</v>
       </c>
@@ -2157,26 +2189,30 @@
         <v>104</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="G28" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G28" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H28" s="8"/>
       <c r="I28" s="14" t="str">
         <f aca="false">IF(AND(G28&lt;&gt;"",H28&lt;&gt;""),H28-G28+1,"")</f>
         <v/>
       </c>
-      <c r="J28" s="10"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J28" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="n">
         <v>3</v>
       </c>
@@ -2184,24 +2220,28 @@
         <v>104</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="G29" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G29" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H29" s="8"/>
       <c r="I29" s="14" t="str">
         <f aca="false">IF(AND(G29&lt;&gt;"",H29&lt;&gt;""),H29-G29+1,"")</f>
         <v/>
       </c>
-      <c r="J29" s="10"/>
+      <c r="J29" s="10" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="n">
@@ -2211,16 +2251,16 @@
         <v>104</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G30" s="8"/>
       <c r="H30" s="8"/>
@@ -2229,7 +2269,7 @@
         <v/>
       </c>
       <c r="J30" s="10" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2240,16 +2280,16 @@
         <v>104</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="E31" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="F31" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>99</v>
       </c>
       <c r="G31" s="8"/>
       <c r="H31" s="8"/>
@@ -2258,7 +2298,7 @@
         <v/>
       </c>
       <c r="J31" s="10" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2269,16 +2309,16 @@
         <v>104</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G32" s="8"/>
       <c r="H32" s="8"/>
@@ -2296,16 +2336,16 @@
         <v>104</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G33" s="8"/>
       <c r="H33" s="8"/>
@@ -2315,78 +2355,86 @@
       </c>
       <c r="J33" s="10"/>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="G34" s="8"/>
+        <v>16</v>
+      </c>
+      <c r="G34" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H34" s="8"/>
       <c r="I34" s="9" t="str">
         <f aca="false">IF(AND(G34&lt;&gt;"",H34&lt;&gt;""),H34-G34+1,"")</f>
         <v/>
       </c>
-      <c r="J34" s="10"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J34" s="10" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="G35" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G35" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H35" s="8"/>
       <c r="I35" s="9" t="str">
         <f aca="false">IF(AND(G35&lt;&gt;"",H35&lt;&gt;""),H35-G35+1,"")</f>
         <v/>
       </c>
-      <c r="J35" s="10"/>
+      <c r="J35" s="10" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G36" s="8"/>
       <c r="H36" s="8"/>
@@ -2395,81 +2443,89 @@
         <v/>
       </c>
       <c r="J36" s="10" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="G37" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G37" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H37" s="8"/>
       <c r="I37" s="9" t="str">
         <f aca="false">IF(AND(G37&lt;&gt;"",H37&lt;&gt;""),H37-G37+1,"")</f>
         <v/>
       </c>
-      <c r="J37" s="10"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J37" s="10" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="G38" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G38" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H38" s="8"/>
       <c r="I38" s="9" t="str">
         <f aca="false">IF(AND(G38&lt;&gt;"",H38&lt;&gt;""),H38-G38+1,"")</f>
         <v/>
       </c>
-      <c r="J38" s="10"/>
+      <c r="J38" s="10" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G39" s="8"/>
       <c r="H39" s="8"/>
@@ -2484,19 +2540,19 @@
         <v>5</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G40" s="8"/>
       <c r="H40" s="8"/>
@@ -2511,19 +2567,19 @@
         <v>5</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G41" s="8"/>
       <c r="H41" s="8"/>
@@ -2538,19 +2594,19 @@
         <v>5</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G42" s="8"/>
       <c r="H42" s="8"/>
@@ -2565,16 +2621,16 @@
         <v>5</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="F43" s="7" t="s">
         <v>28</v>
@@ -2588,7 +2644,7 @@
         <v/>
       </c>
       <c r="J43" s="10" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2596,16 +2652,16 @@
         <v>5</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="D44" s="12" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="E44" s="12" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="F44" s="7" t="s">
         <v>28</v>
@@ -2619,7 +2675,7 @@
         <v/>
       </c>
       <c r="J44" s="10" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2627,16 +2683,16 @@
         <v>5</v>
       </c>
       <c r="B45" s="12" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D45" s="12" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="E45" s="12" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="F45" s="7" t="s">
         <v>28</v>
@@ -2650,7 +2706,7 @@
         <v/>
       </c>
       <c r="J45" s="10" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2658,16 +2714,16 @@
         <v>5</v>
       </c>
       <c r="B46" s="12" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="D46" s="12" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="E46" s="12" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="F46" s="7" t="s">
         <v>28</v>
@@ -2681,7 +2737,7 @@
         <v/>
       </c>
       <c r="J46" s="10" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2689,16 +2745,16 @@
         <v>5</v>
       </c>
       <c r="B47" s="12" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="E47" s="12" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="F47" s="7" t="s">
         <v>28</v>
@@ -2712,7 +2768,7 @@
         <v/>
       </c>
       <c r="J47" s="10" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2720,16 +2776,16 @@
         <v>5</v>
       </c>
       <c r="B48" s="12" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="D48" s="12" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="E48" s="12" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="F48" s="7" t="s">
         <v>28</v>
@@ -2743,7 +2799,7 @@
         <v/>
       </c>
       <c r="J48" s="10" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2751,16 +2807,16 @@
         <v>5</v>
       </c>
       <c r="B49" s="12" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="D49" s="12" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="E49" s="12" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="F49" s="7" t="s">
         <v>28</v>
@@ -2774,7 +2830,7 @@
         <v/>
       </c>
       <c r="J49" s="10" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2782,19 +2838,19 @@
         <v>5</v>
       </c>
       <c r="B50" s="12" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="F50" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G50" s="8"/>
       <c r="H50" s="8"/>
@@ -2809,19 +2865,19 @@
         <v>6</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G51" s="8"/>
       <c r="H51" s="8"/>
@@ -2836,19 +2892,19 @@
         <v>6</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="F52" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G52" s="8"/>
       <c r="H52" s="8"/>
@@ -2863,19 +2919,19 @@
         <v>6</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G53" s="8"/>
       <c r="H53" s="8"/>
@@ -2890,19 +2946,19 @@
         <v>6</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="F54" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G54" s="8"/>
       <c r="H54" s="8"/>
@@ -2917,19 +2973,19 @@
         <v>6</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G55" s="8"/>
       <c r="H55" s="8"/>
@@ -2944,19 +3000,19 @@
         <v>7</v>
       </c>
       <c r="B56" s="12" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="D56" s="12" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="E56" s="12" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="F56" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G56" s="8"/>
       <c r="H56" s="8"/>
@@ -2971,19 +3027,19 @@
         <v>7</v>
       </c>
       <c r="B57" s="12" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G57" s="8"/>
       <c r="H57" s="8"/>
@@ -2992,7 +3048,7 @@
         <v/>
       </c>
       <c r="J57" s="10" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3000,19 +3056,19 @@
         <v>7</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="D58" s="12" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="E58" s="12" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="F58" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G58" s="8"/>
       <c r="H58" s="8"/>
@@ -3027,19 +3083,19 @@
         <v>7</v>
       </c>
       <c r="B59" s="12" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="E59" s="12" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G59" s="8"/>
       <c r="H59" s="8"/>
@@ -3054,19 +3110,19 @@
         <v>7</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="D60" s="12" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="E60" s="12" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G60" s="8"/>
       <c r="H60" s="8"/>
@@ -3081,19 +3137,19 @@
         <v>7</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C61" s="13" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="E61" s="12" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="F61" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G61" s="8"/>
       <c r="H61" s="8"/>
@@ -3108,19 +3164,19 @@
         <v>7</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="D62" s="12" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="E62" s="12" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G62" s="8"/>
       <c r="H62" s="8"/>
@@ -3188,7 +3244,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3199,7 +3255,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>16</v>
@@ -3208,19 +3264,19 @@
         <v>28</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3320,7 +3376,7 @@
       </c>
       <c r="E6" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A6,Plan!$F$5:$F$262,"In progress")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F6" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A6,Plan!$F$5:$F$262,"Blocked")</f>
@@ -3328,7 +3384,7 @@
       </c>
       <c r="G6" s="15" t="n">
         <f aca="false">C6-D6-E6-F6</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" s="16" t="n">
         <f aca="false">IF(C6=0,0,D6/C6)</f>
@@ -3360,7 +3416,7 @@
       </c>
       <c r="E7" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A7,Plan!$F$5:$F$262,"In progress")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F7" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A7,Plan!$F$5:$F$262,"Blocked")</f>
@@ -3368,15 +3424,15 @@
       </c>
       <c r="G7" s="15" t="n">
         <f aca="false">C7-D7-E7-F7</f>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H7" s="16" t="n">
         <f aca="false">IF(C7=0,0,D7/C7)</f>
         <v>0</v>
       </c>
-      <c r="I7" s="17" t="str">
+      <c r="I7" s="17" t="n">
         <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A7)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A7))</f>
-        <v/>
+        <v>46317</v>
       </c>
       <c r="J7" s="17" t="str">
         <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A7)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A7))</f>
@@ -3388,7 +3444,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C8" s="15" t="n">
         <f aca="false">COUNTIF(Plan!$A$5:$A$262,A8)</f>
@@ -3396,11 +3452,11 @@
       </c>
       <c r="D8" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A8,Plan!$F$5:$F$262,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A8,Plan!$F$5:$F$262,"In progress")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F8" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A8,Plan!$F$5:$F$262,"Blocked")</f>
@@ -3408,15 +3464,15 @@
       </c>
       <c r="G8" s="15" t="n">
         <f aca="false">C8-D8-E8-F8</f>
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H8" s="16" t="n">
         <f aca="false">IF(C8=0,0,D8/C8)</f>
-        <v>0</v>
-      </c>
-      <c r="I8" s="17" t="str">
+        <v>0.166666666666667</v>
+      </c>
+      <c r="I8" s="17" t="n">
         <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A8)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A8))</f>
-        <v/>
+        <v>46317</v>
       </c>
       <c r="J8" s="17" t="str">
         <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A8)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A8))</f>
@@ -3428,7 +3484,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C9" s="15" t="n">
         <f aca="false">COUNTIF(Plan!$A$5:$A$262,A9)</f>
@@ -3468,7 +3524,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C10" s="15" t="n">
         <f aca="false">COUNTIF(Plan!$A$5:$A$262,A10)</f>
@@ -3508,7 +3564,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C11" s="15" t="n">
         <f aca="false">COUNTIF(Plan!$A$5:$A$262,A11)</f>
@@ -3546,7 +3602,7 @@
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18"/>
       <c r="B12" s="18" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="C12" s="18" t="n">
         <f aca="false">SUM(C4:C11)</f>
@@ -3554,11 +3610,11 @@
       </c>
       <c r="D12" s="18" t="n">
         <f aca="false">SUM(D4:D11)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E12" s="18" t="n">
         <f aca="false">SUM(E4:E11)</f>
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F12" s="18" t="n">
         <f aca="false">SUM(F4:F11)</f>
@@ -3566,18 +3622,18 @@
       </c>
       <c r="G12" s="18" t="n">
         <f aca="false">SUM(G4:G11)</f>
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="H12" s="19" t="n">
         <f aca="false">IF(C12=0,0,D12/C12)</f>
-        <v>0.224137931034483</v>
+        <v>0.241379310344828</v>
       </c>
       <c r="I12" s="18"/>
       <c r="J12" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -3590,7 +3646,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{57AB1910-F5DB-40D9-BF32-B9C2748016F2}</x14:id>
+          <x14:id>{12FEC671-1068-4164-B43E-E03610888B23}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3606,7 +3662,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{57AB1910-F5DB-40D9-BF32-B9C2748016F2}">
+          <x14:cfRule type="dataBar" id="{12FEC671-1068-4164-B43E-E03610888B23}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
Email alerts: outbox, Alerts page, header bell, Resend sender
- 0021_alerts.sql: notifications outbox filled by triggers (orders, payments, listing review, shop approval, messages), Featured/ad ending reminders, email on/off switch, service-only send RPCs, admin status
- supabase/functions/send-alerts: Edge Function that emails pending alerts through Resend
- alerts.html, header bell with unread count, links in footer, account page, Seller Center and sell page; admin dashboard email status line

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="246">
   <si>
     <t xml:space="preserve">RGBKart Marketplace – Project Plan</t>
   </si>
@@ -357,7 +357,7 @@
     <t xml:space="preserve">Buyers message sellers about a product; both reply on the Messages page</t>
   </si>
   <si>
-    <t xml:space="preserve">Built 22 Oct (messages.html, contact_messages.sql). Only buyer and seller can read a chat. Email/SMS alerts for new messages still to do</t>
+    <t xml:space="preserve">Built 22 Oct (messages.html, contact_messages.sql). Only buyer and seller can read a chat. 23 Oct: email alert for new messages (max one per chat every 30 minutes)</t>
   </si>
   <si>
     <t xml:space="preserve">Checkout &amp; Payments</t>
@@ -444,6 +444,9 @@
     <t xml:space="preserve">Email/SMS receipt after order</t>
   </si>
   <si>
+    <t xml:space="preserve">23 Oct: email to the customer (if they gave an email) and the shop for each order and each status change (0021_alerts.sql). Goes live once Resend is set up. SMS later</t>
+  </si>
+  <si>
     <t xml:space="preserve">Orders &amp; Delivery</t>
   </si>
   <si>
@@ -658,6 +661,9 @@
   </si>
   <si>
     <t xml:space="preserve">Email, SMS and in-app alerts for orders and approvals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 Oct: Alerts page + header bell + email via Resend for orders, payments, listing review, shop approval, messages, Featured/ad ending soon. Each person can switch emails off. SMS later</t>
   </si>
   <si>
     <t xml:space="preserve">6.3</t>
@@ -2136,15 +2142,17 @@
         <v>102</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="G26" s="8" t="n">
         <v>46317</v>
       </c>
-      <c r="H26" s="8"/>
-      <c r="I26" s="9" t="str">
+      <c r="H26" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I26" s="9" t="n">
         <f aca="false">IF(AND(G26&lt;&gt;"",H26&lt;&gt;""),H26-G26+1,"")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J26" s="10" t="s">
         <v>103</v>
@@ -2328,7 +2336,7 @@
       </c>
       <c r="J32" s="10"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="n">
         <v>3</v>
       </c>
@@ -2345,31 +2353,35 @@
         <v>131</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="G33" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H33" s="8"/>
       <c r="I33" s="14" t="str">
         <f aca="false">IF(AND(G33&lt;&gt;"",H33&lt;&gt;""),H33-G33+1,"")</f>
         <v/>
       </c>
-      <c r="J33" s="10"/>
+      <c r="J33" s="10" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F34" s="7" t="s">
         <v>16</v>
@@ -2383,7 +2395,7 @@
         <v/>
       </c>
       <c r="J34" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2391,16 +2403,16 @@
         <v>4</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F35" s="7" t="s">
         <v>28</v>
@@ -2414,7 +2426,7 @@
         <v/>
       </c>
       <c r="J35" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2422,16 +2434,16 @@
         <v>4</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F36" s="7" t="s">
         <v>120</v>
@@ -2443,7 +2455,7 @@
         <v/>
       </c>
       <c r="J36" s="10" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2451,16 +2463,16 @@
         <v>4</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F37" s="7" t="s">
         <v>28</v>
@@ -2474,7 +2486,7 @@
         <v/>
       </c>
       <c r="J37" s="10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2482,16 +2494,16 @@
         <v>4</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F38" s="7" t="s">
         <v>28</v>
@@ -2505,7 +2517,7 @@
         <v/>
       </c>
       <c r="J38" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2513,16 +2525,16 @@
         <v>4</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F39" s="7" t="s">
         <v>120</v>
@@ -2540,16 +2552,16 @@
         <v>5</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F40" s="7" t="s">
         <v>120</v>
@@ -2567,16 +2579,16 @@
         <v>5</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F41" s="7" t="s">
         <v>120</v>
@@ -2594,16 +2606,16 @@
         <v>5</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F42" s="7" t="s">
         <v>120</v>
@@ -2621,16 +2633,16 @@
         <v>5</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F43" s="7" t="s">
         <v>28</v>
@@ -2644,7 +2656,7 @@
         <v/>
       </c>
       <c r="J43" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2652,16 +2664,16 @@
         <v>5</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D44" s="12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E44" s="12" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F44" s="7" t="s">
         <v>28</v>
@@ -2675,7 +2687,7 @@
         <v/>
       </c>
       <c r="J44" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2683,16 +2695,16 @@
         <v>5</v>
       </c>
       <c r="B45" s="12" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D45" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E45" s="12" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F45" s="7" t="s">
         <v>28</v>
@@ -2706,7 +2718,7 @@
         <v/>
       </c>
       <c r="J45" s="10" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2714,16 +2726,16 @@
         <v>5</v>
       </c>
       <c r="B46" s="12" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D46" s="12" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E46" s="12" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F46" s="7" t="s">
         <v>28</v>
@@ -2737,7 +2749,7 @@
         <v/>
       </c>
       <c r="J46" s="10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2745,16 +2757,16 @@
         <v>5</v>
       </c>
       <c r="B47" s="12" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E47" s="12" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F47" s="7" t="s">
         <v>28</v>
@@ -2768,7 +2780,7 @@
         <v/>
       </c>
       <c r="J47" s="10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2776,16 +2788,16 @@
         <v>5</v>
       </c>
       <c r="B48" s="12" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D48" s="12" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E48" s="12" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F48" s="7" t="s">
         <v>28</v>
@@ -2799,7 +2811,7 @@
         <v/>
       </c>
       <c r="J48" s="10" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2807,16 +2819,16 @@
         <v>5</v>
       </c>
       <c r="B49" s="12" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D49" s="12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E49" s="12" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F49" s="7" t="s">
         <v>28</v>
@@ -2830,7 +2842,7 @@
         <v/>
       </c>
       <c r="J49" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2838,16 +2850,16 @@
         <v>5</v>
       </c>
       <c r="B50" s="12" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F50" s="7" t="s">
         <v>120</v>
@@ -2865,16 +2877,16 @@
         <v>6</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F51" s="7" t="s">
         <v>120</v>
@@ -2887,48 +2899,52 @@
       </c>
       <c r="J51" s="10"/>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="n">
         <v>6</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F52" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="G52" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G52" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H52" s="8"/>
       <c r="I52" s="9" t="str">
         <f aca="false">IF(AND(G52&lt;&gt;"",H52&lt;&gt;""),H52-G52+1,"")</f>
         <v/>
       </c>
-      <c r="J52" s="10"/>
+      <c r="J52" s="10" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="n">
         <v>6</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F53" s="7" t="s">
         <v>120</v>
@@ -2946,16 +2962,16 @@
         <v>6</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F54" s="7" t="s">
         <v>120</v>
@@ -2973,16 +2989,16 @@
         <v>6</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="F55" s="7" t="s">
         <v>120</v>
@@ -3000,16 +3016,16 @@
         <v>7</v>
       </c>
       <c r="B56" s="12" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D56" s="12" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E56" s="12" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F56" s="7" t="s">
         <v>120</v>
@@ -3027,16 +3043,16 @@
         <v>7</v>
       </c>
       <c r="B57" s="12" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F57" s="7" t="s">
         <v>120</v>
@@ -3048,7 +3064,7 @@
         <v/>
       </c>
       <c r="J57" s="10" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3056,16 +3072,16 @@
         <v>7</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D58" s="12" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E58" s="12" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="F58" s="7" t="s">
         <v>120</v>
@@ -3083,16 +3099,16 @@
         <v>7</v>
       </c>
       <c r="B59" s="12" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="E59" s="12" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F59" s="7" t="s">
         <v>120</v>
@@ -3110,16 +3126,16 @@
         <v>7</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D60" s="12" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E60" s="12" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F60" s="7" t="s">
         <v>120</v>
@@ -3137,16 +3153,16 @@
         <v>7</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C61" s="13" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E61" s="12" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F61" s="7" t="s">
         <v>120</v>
@@ -3164,16 +3180,16 @@
         <v>7</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D62" s="12" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E62" s="12" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F62" s="7" t="s">
         <v>120</v>
@@ -3244,7 +3260,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3255,7 +3271,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>16</v>
@@ -3264,19 +3280,19 @@
         <v>28</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>120</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3372,11 +3388,11 @@
       </c>
       <c r="D6" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A6,Plan!$F$5:$F$262,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A6,Plan!$F$5:$F$262,"In progress")</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F6" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A6,Plan!$F$5:$F$262,"Blocked")</f>
@@ -3388,15 +3404,15 @@
       </c>
       <c r="H6" s="16" t="n">
         <f aca="false">IF(C6=0,0,D6/C6)</f>
-        <v>0</v>
+        <v>0.142857142857143</v>
       </c>
       <c r="I6" s="17" t="n">
         <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A6)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A6))</f>
         <v>46317</v>
       </c>
-      <c r="J6" s="17" t="str">
+      <c r="J6" s="17" t="n">
         <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A6)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A6))</f>
-        <v/>
+        <v>46317</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3416,7 +3432,7 @@
       </c>
       <c r="E7" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A7,Plan!$F$5:$F$262,"In progress")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F7" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A7,Plan!$F$5:$F$262,"Blocked")</f>
@@ -3424,7 +3440,7 @@
       </c>
       <c r="G7" s="15" t="n">
         <f aca="false">C7-D7-E7-F7</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H7" s="16" t="n">
         <f aca="false">IF(C7=0,0,D7/C7)</f>
@@ -3444,7 +3460,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C8" s="15" t="n">
         <f aca="false">COUNTIF(Plan!$A$5:$A$262,A8)</f>
@@ -3484,7 +3500,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C9" s="15" t="n">
         <f aca="false">COUNTIF(Plan!$A$5:$A$262,A9)</f>
@@ -3524,7 +3540,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C10" s="15" t="n">
         <f aca="false">COUNTIF(Plan!$A$5:$A$262,A10)</f>
@@ -3536,7 +3552,7 @@
       </c>
       <c r="E10" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A10,Plan!$F$5:$F$262,"In progress")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A10,Plan!$F$5:$F$262,"Blocked")</f>
@@ -3544,15 +3560,15 @@
       </c>
       <c r="G10" s="15" t="n">
         <f aca="false">C10-D10-E10-F10</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H10" s="16" t="n">
         <f aca="false">IF(C10=0,0,D10/C10)</f>
         <v>0</v>
       </c>
-      <c r="I10" s="17" t="str">
+      <c r="I10" s="17" t="n">
         <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A10)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A10))</f>
-        <v/>
+        <v>46317</v>
       </c>
       <c r="J10" s="17" t="str">
         <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A10)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A10))</f>
@@ -3564,7 +3580,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C11" s="15" t="n">
         <f aca="false">COUNTIF(Plan!$A$5:$A$262,A11)</f>
@@ -3602,7 +3618,7 @@
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18"/>
       <c r="B12" s="18" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C12" s="18" t="n">
         <f aca="false">SUM(C4:C11)</f>
@@ -3610,11 +3626,11 @@
       </c>
       <c r="D12" s="18" t="n">
         <f aca="false">SUM(D4:D11)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E12" s="18" t="n">
         <f aca="false">SUM(E4:E11)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F12" s="18" t="n">
         <f aca="false">SUM(F4:F11)</f>
@@ -3622,18 +3638,18 @@
       </c>
       <c r="G12" s="18" t="n">
         <f aca="false">SUM(G4:G11)</f>
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H12" s="19" t="n">
         <f aca="false">IF(C12=0,0,D12/C12)</f>
-        <v>0.241379310344828</v>
+        <v>0.258620689655172</v>
       </c>
       <c r="I12" s="18"/>
       <c r="J12" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>
@@ -3646,7 +3662,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{12FEC671-1068-4164-B43E-E03610888B23}</x14:id>
+          <x14:id>{199BC88C-56E1-44F4-8DDC-2F3DB58232EB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3662,7 +3678,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{12FEC671-1068-4164-B43E-E03610888B23}">
+          <x14:cfRule type="dataBar" id="{199BC88C-56E1-44F4-8DDC-2F3DB58232EB}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
English / Bangla: language switch and Bangla shop pages
- 0022_bangla.sql: Bangla names for categories (pre-filled), products, shops and home sections; Bangla edits send a live product back for review; admin_set_product_bangla
- site/i18n.js: language choice, dictionary and patterns, translates page text as it appears, Bangla digits and dates, Hind Siliguri sizing
- shopper pages, cart and menu show Bangla names; switch in menu bar, footer, sign-in and sell pages
- Bangla name fields in Admin (categories, home sections, add product), Seller Center (product, shop name) and the sell form

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Plan!$A$4:$J$62</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Plan!$A$4:$J$63</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="250">
   <si>
     <t xml:space="preserve">RGBKart Marketplace – Project Plan</t>
   </si>
@@ -358,6 +358,18 @@
   </si>
   <si>
     <t xml:space="preserve">Built 22 Oct (messages.html, contact_messages.sql). Only buyer and seller can read a chat. 23 Oct: email alert for new messages (max one per chat every 30 minutes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">English / Bangla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Language switch; shop pages, names of categories, products and shops in Bangla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 Oct: i18n.js translates shopper pages (home, categories, browse, product, cart, checkout, orders, messages, alerts, sign-in, sell) with Bangla digits; Bangla name fields for categories, products, shops, home sections (0022_bangla.sql). Seller Center and Admin still English</t>
   </si>
   <si>
     <t xml:space="preserve">Checkout &amp; Payments</t>
@@ -1386,7 +1398,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J62"/>
+  <dimension ref="A1:J63"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -2158,21 +2170,21 @@
         <v>103</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B27" s="12" t="s">
+    <row r="27" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="D27" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="D27" s="12" t="s">
+      <c r="E27" s="5" t="s">
         <v>106</v>
-      </c>
-      <c r="E27" s="12" t="s">
-        <v>107</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>28</v>
@@ -2181,20 +2193,20 @@
         <v>46317</v>
       </c>
       <c r="H27" s="8"/>
-      <c r="I27" s="14" t="str">
+      <c r="I27" s="9" t="str">
         <f aca="false">IF(AND(G27&lt;&gt;"",H27&lt;&gt;""),H27-G27+1,"")</f>
         <v/>
       </c>
       <c r="J27" s="10" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="n">
         <v>3</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C28" s="13" t="s">
         <v>109</v>
@@ -2220,12 +2232,12 @@
         <v>112</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="n">
         <v>3</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C29" s="13" t="s">
         <v>113</v>
@@ -2251,12 +2263,12 @@
         <v>116</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="n">
         <v>3</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C30" s="13" t="s">
         <v>117</v>
@@ -2268,16 +2280,18 @@
         <v>119</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="G30" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G30" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H30" s="8"/>
       <c r="I30" s="14" t="str">
         <f aca="false">IF(AND(G30&lt;&gt;"",H30&lt;&gt;""),H30-G30+1,"")</f>
         <v/>
       </c>
       <c r="J30" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2285,19 +2299,19 @@
         <v>3</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C31" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="D31" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="D31" s="12" t="s">
+      <c r="E31" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="E31" s="12" t="s">
+      <c r="F31" s="7" t="s">
         <v>124</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>120</v>
       </c>
       <c r="G31" s="8"/>
       <c r="H31" s="8"/>
@@ -2314,7 +2328,7 @@
         <v>3</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C32" s="13" t="s">
         <v>126</v>
@@ -2326,7 +2340,7 @@
         <v>128</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G32" s="8"/>
       <c r="H32" s="8"/>
@@ -2334,68 +2348,66 @@
         <f aca="false">IF(AND(G32&lt;&gt;"",H32&lt;&gt;""),H32-G32+1,"")</f>
         <v/>
       </c>
-      <c r="J32" s="10"/>
-    </row>
-    <row r="33" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J32" s="10" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="n">
         <v>3</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="G33" s="8" t="n">
-        <v>46317</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="G33" s="8"/>
       <c r="H33" s="8"/>
       <c r="I33" s="14" t="str">
         <f aca="false">IF(AND(G33&lt;&gt;"",H33&lt;&gt;""),H33-G33+1,"")</f>
         <v/>
       </c>
-      <c r="J33" s="10" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B34" s="5" t="s">
+      <c r="J33" s="10"/>
+    </row>
+    <row r="34" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C34" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="D34" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="E34" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="E34" s="5" t="s">
+      <c r="F34" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G34" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H34" s="8"/>
+      <c r="I34" s="14" t="str">
+        <f aca="false">IF(AND(G34&lt;&gt;"",H34&lt;&gt;""),H34-G34+1,"")</f>
+        <v/>
+      </c>
+      <c r="J34" s="10" t="s">
         <v>136</v>
-      </c>
-      <c r="F34" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G34" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H34" s="8"/>
-      <c r="I34" s="9" t="str">
-        <f aca="false">IF(AND(G34&lt;&gt;"",H34&lt;&gt;""),H34-G34+1,"")</f>
-        <v/>
-      </c>
-      <c r="J34" s="10" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2403,7 +2415,7 @@
         <v>4</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>138</v>
@@ -2415,7 +2427,7 @@
         <v>140</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="G35" s="8" t="n">
         <v>46317</v>
@@ -2429,12 +2441,12 @@
         <v>141</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>142</v>
@@ -2446,9 +2458,11 @@
         <v>144</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="G36" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G36" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H36" s="8"/>
       <c r="I36" s="9" t="str">
         <f aca="false">IF(AND(G36&lt;&gt;"",H36&lt;&gt;""),H36-G36+1,"")</f>
@@ -2458,12 +2472,12 @@
         <v>145</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>146</v>
@@ -2475,11 +2489,9 @@
         <v>148</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="G37" s="8" t="n">
-        <v>46317</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="G37" s="8"/>
       <c r="H37" s="8"/>
       <c r="I37" s="9" t="str">
         <f aca="false">IF(AND(G37&lt;&gt;"",H37&lt;&gt;""),H37-G37+1,"")</f>
@@ -2494,7 +2506,7 @@
         <v>4</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>150</v>
@@ -2520,12 +2532,12 @@
         <v>153</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>154</v>
@@ -2537,38 +2549,42 @@
         <v>156</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="G39" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G39" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H39" s="8"/>
       <c r="I39" s="9" t="str">
         <f aca="false">IF(AND(G39&lt;&gt;"",H39&lt;&gt;""),H39-G39+1,"")</f>
         <v/>
       </c>
-      <c r="J39" s="10"/>
-    </row>
-    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="B40" s="12" t="s">
+      <c r="J39" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="C40" s="13" t="s">
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C40" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="D40" s="12" t="s">
+      <c r="D40" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="E40" s="12" t="s">
+      <c r="E40" s="5" t="s">
         <v>160</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G40" s="8"/>
       <c r="H40" s="8"/>
-      <c r="I40" s="14" t="str">
+      <c r="I40" s="9" t="str">
         <f aca="false">IF(AND(G40&lt;&gt;"",H40&lt;&gt;""),H40-G40+1,"")</f>
         <v/>
       </c>
@@ -2579,19 +2595,19 @@
         <v>5</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G41" s="8"/>
       <c r="H41" s="8"/>
@@ -2606,19 +2622,19 @@
         <v>5</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G42" s="8"/>
       <c r="H42" s="8"/>
@@ -2628,43 +2644,39 @@
       </c>
       <c r="J42" s="10"/>
     </row>
-    <row r="43" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="n">
         <v>5</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="G43" s="8" t="n">
-        <v>46317</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="G43" s="8"/>
       <c r="H43" s="8"/>
       <c r="I43" s="14" t="str">
         <f aca="false">IF(AND(G43&lt;&gt;"",H43&lt;&gt;""),H43-G43+1,"")</f>
         <v/>
       </c>
-      <c r="J43" s="10" t="s">
-        <v>170</v>
-      </c>
+      <c r="J43" s="10"/>
     </row>
     <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="11" t="n">
         <v>5</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C44" s="13" t="s">
         <v>171</v>
@@ -2695,7 +2707,7 @@
         <v>5</v>
       </c>
       <c r="B45" s="12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C45" s="13" t="s">
         <v>175</v>
@@ -2721,12 +2733,12 @@
         <v>178</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="11" t="n">
         <v>5</v>
       </c>
       <c r="B46" s="12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C46" s="13" t="s">
         <v>179</v>
@@ -2752,12 +2764,12 @@
         <v>182</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="n">
         <v>5</v>
       </c>
       <c r="B47" s="12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C47" s="13" t="s">
         <v>183</v>
@@ -2783,12 +2795,12 @@
         <v>186</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="11" t="n">
         <v>5</v>
       </c>
       <c r="B48" s="12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C48" s="13" t="s">
         <v>187</v>
@@ -2814,12 +2826,12 @@
         <v>190</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="n">
         <v>5</v>
       </c>
       <c r="B49" s="12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C49" s="13" t="s">
         <v>191</v>
@@ -2845,12 +2857,12 @@
         <v>194</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="n">
         <v>5</v>
       </c>
       <c r="B50" s="12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C50" s="13" t="s">
         <v>195</v>
@@ -2862,80 +2874,80 @@
         <v>197</v>
       </c>
       <c r="F50" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="G50" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G50" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H50" s="8"/>
       <c r="I50" s="14" t="str">
         <f aca="false">IF(AND(G50&lt;&gt;"",H50&lt;&gt;""),H50-G50+1,"")</f>
         <v/>
       </c>
-      <c r="J50" s="10"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B51" s="5" t="s">
+      <c r="J50" s="10" t="s">
         <v>198</v>
       </c>
-      <c r="C51" s="6" t="s">
+    </row>
+    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B51" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="C51" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="D51" s="5" t="s">
+      <c r="D51" s="12" t="s">
         <v>200</v>
       </c>
-      <c r="E51" s="5" t="s">
+      <c r="E51" s="12" t="s">
         <v>201</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G51" s="8"/>
       <c r="H51" s="8"/>
-      <c r="I51" s="9" t="str">
+      <c r="I51" s="14" t="str">
         <f aca="false">IF(AND(G51&lt;&gt;"",H51&lt;&gt;""),H51-G51+1,"")</f>
         <v/>
       </c>
       <c r="J51" s="10"/>
     </row>
-    <row r="52" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="n">
         <v>6</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F52" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="G52" s="8" t="n">
-        <v>46317</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="G52" s="8"/>
       <c r="H52" s="8"/>
       <c r="I52" s="9" t="str">
         <f aca="false">IF(AND(G52&lt;&gt;"",H52&lt;&gt;""),H52-G52+1,"")</f>
         <v/>
       </c>
-      <c r="J52" s="10" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J52" s="10"/>
+    </row>
+    <row r="53" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="n">
         <v>6</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>206</v>
@@ -2947,34 +2959,38 @@
         <v>208</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="G53" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G53" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="H53" s="8"/>
       <c r="I53" s="9" t="str">
         <f aca="false">IF(AND(G53&lt;&gt;"",H53&lt;&gt;""),H53-G53+1,"")</f>
         <v/>
       </c>
-      <c r="J53" s="10"/>
+      <c r="J53" s="10" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="n">
         <v>6</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F54" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G54" s="8"/>
       <c r="H54" s="8"/>
@@ -2989,19 +3005,19 @@
         <v>6</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G55" s="8"/>
       <c r="H55" s="8"/>
@@ -3012,27 +3028,27 @@
       <c r="J55" s="10"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="B56" s="12" t="s">
-        <v>215</v>
-      </c>
-      <c r="C56" s="13" t="s">
+      <c r="A56" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="C56" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="D56" s="12" t="s">
+      <c r="D56" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="E56" s="12" t="s">
+      <c r="E56" s="5" t="s">
         <v>218</v>
       </c>
       <c r="F56" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G56" s="8"/>
       <c r="H56" s="8"/>
-      <c r="I56" s="14" t="str">
+      <c r="I56" s="9" t="str">
         <f aca="false">IF(AND(G56&lt;&gt;"",H56&lt;&gt;""),H56-G56+1,"")</f>
         <v/>
       </c>
@@ -3043,19 +3059,19 @@
         <v>7</v>
       </c>
       <c r="B57" s="12" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G57" s="8"/>
       <c r="H57" s="8"/>
@@ -3063,16 +3079,14 @@
         <f aca="false">IF(AND(G57&lt;&gt;"",H57&lt;&gt;""),H57-G57+1,"")</f>
         <v/>
       </c>
-      <c r="J57" s="10" t="s">
-        <v>222</v>
-      </c>
+      <c r="J57" s="10"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="n">
         <v>7</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C58" s="13" t="s">
         <v>223</v>
@@ -3084,7 +3098,7 @@
         <v>225</v>
       </c>
       <c r="F58" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G58" s="8"/>
       <c r="H58" s="8"/>
@@ -3092,26 +3106,28 @@
         <f aca="false">IF(AND(G58&lt;&gt;"",H58&lt;&gt;""),H58-G58+1,"")</f>
         <v/>
       </c>
-      <c r="J58" s="10"/>
+      <c r="J58" s="10" t="s">
+        <v>226</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="n">
         <v>7</v>
       </c>
       <c r="B59" s="12" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E59" s="12" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G59" s="8"/>
       <c r="H59" s="8"/>
@@ -3126,19 +3142,19 @@
         <v>7</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D60" s="12" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E60" s="12" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G60" s="8"/>
       <c r="H60" s="8"/>
@@ -3153,19 +3169,19 @@
         <v>7</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C61" s="13" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E61" s="12" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F61" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G61" s="8"/>
       <c r="H61" s="8"/>
@@ -3180,19 +3196,19 @@
         <v>7</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D62" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E62" s="12" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G62" s="8"/>
       <c r="H62" s="8"/>
@@ -3202,12 +3218,39 @@
       </c>
       <c r="J62" s="10"/>
     </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B63" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="C63" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="D63" s="12" t="s">
+        <v>240</v>
+      </c>
+      <c r="E63" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="F63" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="G63" s="8"/>
+      <c r="H63" s="8"/>
+      <c r="I63" s="14" t="str">
+        <f aca="false">IF(AND(G63&lt;&gt;"",H63&lt;&gt;""),H63-G63+1,"")</f>
+        <v/>
+      </c>
+      <c r="J63" s="10"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J62"/>
+  <autoFilter ref="A4:J63"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F262">
+  <conditionalFormatting sqref="F5:F263">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>$F5="Done"</formula>
     </cfRule>
@@ -3219,11 +3262,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F262" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F263" type="list">
       <formula1>"Not started,In progress,Blocked,Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Enter a date, e.g. 22-Oct-2026" errorStyle="stop" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G5:H262" type="date">
+    <dataValidation allowBlank="true" error="Enter a date, e.g. 22-Oct-2026" errorStyle="stop" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G5:H263" type="date">
       <formula1>DATE(2020,1,1)</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3260,7 +3303,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3271,7 +3314,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>16</v>
@@ -3280,19 +3323,19 @@
         <v>28</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3303,19 +3346,19 @@
         <v>12</v>
       </c>
       <c r="C4" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$262,A4)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$263,A4)</f>
         <v>7</v>
       </c>
       <c r="D4" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A4,Plan!$F$5:$F$262,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A4,Plan!$F$5:$F$263,"Done")</f>
         <v>6</v>
       </c>
       <c r="E4" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A4,Plan!$F$5:$F$262,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A4,Plan!$F$5:$F$263,"In progress")</f>
         <v>1</v>
       </c>
       <c r="F4" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A4,Plan!$F$5:$F$262,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A4,Plan!$F$5:$F$263,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G4" s="15" t="n">
@@ -3327,11 +3370,11 @@
         <v>0.857142857142857</v>
       </c>
       <c r="I4" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A4)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A4))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A4)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A4))</f>
         <v>46317</v>
       </c>
       <c r="J4" s="17" t="n">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A4)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A4))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A4)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A4))</f>
         <v>46317</v>
       </c>
     </row>
@@ -3343,19 +3386,19 @@
         <v>42</v>
       </c>
       <c r="C5" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$262,A5)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$263,A5)</f>
         <v>8</v>
       </c>
       <c r="D5" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A5,Plan!$F$5:$F$262,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A5,Plan!$F$5:$F$263,"Done")</f>
         <v>7</v>
       </c>
       <c r="E5" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A5,Plan!$F$5:$F$262,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A5,Plan!$F$5:$F$263,"In progress")</f>
         <v>1</v>
       </c>
       <c r="F5" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A5,Plan!$F$5:$F$262,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A5,Plan!$F$5:$F$263,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G5" s="15" t="n">
@@ -3367,11 +3410,11 @@
         <v>0.875</v>
       </c>
       <c r="I5" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A5)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A5))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A5)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A5))</f>
         <v>46317</v>
       </c>
       <c r="J5" s="17" t="n">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A5)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A5))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A5)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A5))</f>
         <v>46317</v>
       </c>
     </row>
@@ -3383,19 +3426,19 @@
         <v>75</v>
       </c>
       <c r="C6" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$262,A6)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$263,A6)</f>
+        <v>8</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A6,Plan!$F$5:$F$263,"Done")</f>
+        <v>1</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A6,Plan!$F$5:$F$263,"In progress")</f>
         <v>7</v>
       </c>
-      <c r="D6" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A6,Plan!$F$5:$F$262,"Done")</f>
-        <v>1</v>
-      </c>
-      <c r="E6" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A6,Plan!$F$5:$F$262,"In progress")</f>
-        <v>6</v>
-      </c>
       <c r="F6" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A6,Plan!$F$5:$F$262,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A6,Plan!$F$5:$F$263,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G6" s="15" t="n">
@@ -3404,14 +3447,14 @@
       </c>
       <c r="H6" s="16" t="n">
         <f aca="false">IF(C6=0,0,D6/C6)</f>
-        <v>0.142857142857143</v>
+        <v>0.125</v>
       </c>
       <c r="I6" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A6)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A6))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A6)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A6))</f>
         <v>46317</v>
       </c>
       <c r="J6" s="17" t="n">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A6)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A6))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A6)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A6))</f>
         <v>46317</v>
       </c>
     </row>
@@ -3420,22 +3463,22 @@
         <v>3</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C7" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$262,A7)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$263,A7)</f>
         <v>7</v>
       </c>
       <c r="D7" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A7,Plan!$F$5:$F$262,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A7,Plan!$F$5:$F$263,"Done")</f>
         <v>0</v>
       </c>
       <c r="E7" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A7,Plan!$F$5:$F$262,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A7,Plan!$F$5:$F$263,"In progress")</f>
         <v>4</v>
       </c>
       <c r="F7" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A7,Plan!$F$5:$F$262,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A7,Plan!$F$5:$F$263,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G7" s="15" t="n">
@@ -3447,11 +3490,11 @@
         <v>0</v>
       </c>
       <c r="I7" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A7)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A7))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A7)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A7))</f>
         <v>46317</v>
       </c>
       <c r="J7" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A7)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A7))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A7)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A7))</f>
         <v/>
       </c>
     </row>
@@ -3460,22 +3503,22 @@
         <v>4</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C8" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$262,A8)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$263,A8)</f>
         <v>6</v>
       </c>
       <c r="D8" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A8,Plan!$F$5:$F$262,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A8,Plan!$F$5:$F$263,"Done")</f>
         <v>1</v>
       </c>
       <c r="E8" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A8,Plan!$F$5:$F$262,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A8,Plan!$F$5:$F$263,"In progress")</f>
         <v>3</v>
       </c>
       <c r="F8" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A8,Plan!$F$5:$F$262,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A8,Plan!$F$5:$F$263,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G8" s="15" t="n">
@@ -3487,11 +3530,11 @@
         <v>0.166666666666667</v>
       </c>
       <c r="I8" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A8)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A8))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A8)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A8))</f>
         <v>46317</v>
       </c>
       <c r="J8" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A8)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A8))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A8)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A8))</f>
         <v/>
       </c>
     </row>
@@ -3500,22 +3543,22 @@
         <v>5</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C9" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$262,A9)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$263,A9)</f>
         <v>11</v>
       </c>
       <c r="D9" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A9,Plan!$F$5:$F$262,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A9,Plan!$F$5:$F$263,"Done")</f>
         <v>0</v>
       </c>
       <c r="E9" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A9,Plan!$F$5:$F$262,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A9,Plan!$F$5:$F$263,"In progress")</f>
         <v>7</v>
       </c>
       <c r="F9" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A9,Plan!$F$5:$F$262,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A9,Plan!$F$5:$F$263,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G9" s="15" t="n">
@@ -3527,11 +3570,11 @@
         <v>0</v>
       </c>
       <c r="I9" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A9)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A9))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A9)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A9))</f>
         <v>46317</v>
       </c>
       <c r="J9" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A9)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A9))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A9)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A9))</f>
         <v/>
       </c>
     </row>
@@ -3540,22 +3583,22 @@
         <v>6</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C10" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$262,A10)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$263,A10)</f>
         <v>5</v>
       </c>
       <c r="D10" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A10,Plan!$F$5:$F$262,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A10,Plan!$F$5:$F$263,"Done")</f>
         <v>0</v>
       </c>
       <c r="E10" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A10,Plan!$F$5:$F$262,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A10,Plan!$F$5:$F$263,"In progress")</f>
         <v>1</v>
       </c>
       <c r="F10" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A10,Plan!$F$5:$F$262,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A10,Plan!$F$5:$F$263,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G10" s="15" t="n">
@@ -3567,11 +3610,11 @@
         <v>0</v>
       </c>
       <c r="I10" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A10)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A10))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A10)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A10))</f>
         <v>46317</v>
       </c>
       <c r="J10" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A10)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A10))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A10)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A10))</f>
         <v/>
       </c>
     </row>
@@ -3580,22 +3623,22 @@
         <v>7</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C11" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$262,A11)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$263,A11)</f>
         <v>7</v>
       </c>
       <c r="D11" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A11,Plan!$F$5:$F$262,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A11,Plan!$F$5:$F$263,"Done")</f>
         <v>0</v>
       </c>
       <c r="E11" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A11,Plan!$F$5:$F$262,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A11,Plan!$F$5:$F$263,"In progress")</f>
         <v>0</v>
       </c>
       <c r="F11" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$262,$A11,Plan!$F$5:$F$262,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A11,Plan!$F$5:$F$263,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G11" s="15" t="n">
@@ -3607,22 +3650,22 @@
         <v>0</v>
       </c>
       <c r="I11" s="17" t="str">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A11)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$262,Plan!$A$5:$A$262,A11))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A11)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A11))</f>
         <v/>
       </c>
       <c r="J11" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A11)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$262,Plan!$A$5:$A$262,A11))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A11)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A11))</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18"/>
       <c r="B12" s="18" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="C12" s="18" t="n">
         <f aca="false">SUM(C4:C11)</f>
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D12" s="18" t="n">
         <f aca="false">SUM(D4:D11)</f>
@@ -3630,7 +3673,7 @@
       </c>
       <c r="E12" s="18" t="n">
         <f aca="false">SUM(E4:E11)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F12" s="18" t="n">
         <f aca="false">SUM(F4:F11)</f>
@@ -3642,14 +3685,14 @@
       </c>
       <c r="H12" s="19" t="n">
         <f aca="false">IF(C12=0,0,D12/C12)</f>
-        <v>0.258620689655172</v>
+        <v>0.254237288135593</v>
       </c>
       <c r="I12" s="18"/>
       <c r="J12" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
   </sheetData>
@@ -3662,7 +3705,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{199BC88C-56E1-44F4-8DDC-2F3DB58232EB}</x14:id>
+          <x14:id>{405640DE-A7CB-41B0-B4DB-6B9D1A6464E3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3678,7 +3721,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{199BC88C-56E1-44F4-8DDC-2F3DB58232EB}">
+          <x14:cfRule type="dataBar" id="{405640DE-A7CB-41B0-B4DB-6B9D1A6464E3}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
Plan: email alerts sending pending (7.8); 0022 run
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Plan!$A$4:$J$63</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Plan!$A$4:$J$64</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="254">
   <si>
     <t xml:space="preserve">RGBKart Marketplace – Project Plan</t>
   </si>
@@ -675,7 +675,7 @@
     <t xml:space="preserve">Email, SMS and in-app alerts for orders and approvals</t>
   </si>
   <si>
-    <t xml:space="preserve">23 Oct: Alerts page + header bell + email via Resend for orders, payments, listing review, shop approval, messages, Featured/ad ending soon. Each person can switch emails off. SMS later</t>
+    <t xml:space="preserve">23 Oct: Alerts page + header bell + email via Resend for orders, payments, listing review, shop approval, messages, Featured/ad ending soon. Each person can switch emails off. Email sending pending, see 7.8. SMS later</t>
   </si>
   <si>
     <t xml:space="preserve">6.3</t>
@@ -774,13 +774,25 @@
     <t xml:space="preserve">Launch, monitoring, database backups</t>
   </si>
   <si>
+    <t xml:space="preserve">7.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email alerts (sending)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Send the alerts by email from our own domain through Resend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blocked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PENDING, set up later (owner, 23 Oct): waits for the real domain. Steps: Resend account + domain DNS records in Hostinger; deploy Edge Function send-alerts (in the repo); secrets RESEND_API_KEY, ALERT_FROM, SITE_URL; Supabase Cron every 5 min; first add a rule so only recent alerts are emailed. Alerts already show on the site (0021_alerts.sql run)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Progress by phase</t>
   </si>
   <si>
     <t xml:space="preserve">Sub-phases</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blocked</t>
   </si>
   <si>
     <t xml:space="preserve">% complete</t>
@@ -1036,7 +1048,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="14">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1079,6 +1091,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFF8E3E0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFBEFD5"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
@@ -1104,6 +1124,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF8A5A00"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFA3322A"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1398,7 +1426,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J63"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -3245,28 +3273,57 @@
       </c>
       <c r="J63" s="10"/>
     </row>
+    <row r="64" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B64" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="C64" s="13" t="s">
+        <v>242</v>
+      </c>
+      <c r="D64" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="E64" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="F64" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="G64" s="8"/>
+      <c r="H64" s="8"/>
+      <c r="I64" s="14" t="str">
+        <f aca="false">IF(AND(G64&lt;&gt;"",H64&lt;&gt;""),H64-G64+1,"")</f>
+        <v/>
+      </c>
+      <c r="J64" s="10" t="s">
+        <v>246</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J63"/>
+  <autoFilter ref="A4:J64"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F263">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+  <conditionalFormatting sqref="F5:F264">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>$F5="Done"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>$F5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>$F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F263" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F264" type="list">
       <formula1>"Not started,In progress,Blocked,Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Enter a date, e.g. 22-Oct-2026" errorStyle="stop" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G5:H263" type="date">
+    <dataValidation allowBlank="true" error="Enter a date, e.g. 22-Oct-2026" errorStyle="stop" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G5:H264" type="date">
       <formula1>DATE(2020,1,1)</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3303,7 +3360,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3314,7 +3371,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>16</v>
@@ -3323,19 +3380,19 @@
         <v>28</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>124</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3346,19 +3403,19 @@
         <v>12</v>
       </c>
       <c r="C4" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$263,A4)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$264,A4)</f>
         <v>7</v>
       </c>
       <c r="D4" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A4,Plan!$F$5:$F$263,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A4,Plan!$F$5:$F$264,"Done")</f>
         <v>6</v>
       </c>
       <c r="E4" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A4,Plan!$F$5:$F$263,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A4,Plan!$F$5:$F$264,"In progress")</f>
         <v>1</v>
       </c>
       <c r="F4" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A4,Plan!$F$5:$F$263,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A4,Plan!$F$5:$F$264,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G4" s="15" t="n">
@@ -3370,11 +3427,11 @@
         <v>0.857142857142857</v>
       </c>
       <c r="I4" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A4)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A4))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A4)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A4))</f>
         <v>46317</v>
       </c>
       <c r="J4" s="17" t="n">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A4)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A4))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A4)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A4))</f>
         <v>46317</v>
       </c>
     </row>
@@ -3386,19 +3443,19 @@
         <v>42</v>
       </c>
       <c r="C5" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$263,A5)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$264,A5)</f>
         <v>8</v>
       </c>
       <c r="D5" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A5,Plan!$F$5:$F$263,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A5,Plan!$F$5:$F$264,"Done")</f>
         <v>7</v>
       </c>
       <c r="E5" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A5,Plan!$F$5:$F$263,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A5,Plan!$F$5:$F$264,"In progress")</f>
         <v>1</v>
       </c>
       <c r="F5" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A5,Plan!$F$5:$F$263,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A5,Plan!$F$5:$F$264,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G5" s="15" t="n">
@@ -3410,11 +3467,11 @@
         <v>0.875</v>
       </c>
       <c r="I5" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A5)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A5))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A5)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A5))</f>
         <v>46317</v>
       </c>
       <c r="J5" s="17" t="n">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A5)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A5))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A5)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A5))</f>
         <v>46317</v>
       </c>
     </row>
@@ -3426,19 +3483,19 @@
         <v>75</v>
       </c>
       <c r="C6" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$263,A6)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$264,A6)</f>
         <v>8</v>
       </c>
       <c r="D6" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A6,Plan!$F$5:$F$263,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A6,Plan!$F$5:$F$264,"Done")</f>
         <v>1</v>
       </c>
       <c r="E6" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A6,Plan!$F$5:$F$263,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A6,Plan!$F$5:$F$264,"In progress")</f>
         <v>7</v>
       </c>
       <c r="F6" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A6,Plan!$F$5:$F$263,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A6,Plan!$F$5:$F$264,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G6" s="15" t="n">
@@ -3450,11 +3507,11 @@
         <v>0.125</v>
       </c>
       <c r="I6" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A6)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A6))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A6)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A6))</f>
         <v>46317</v>
       </c>
       <c r="J6" s="17" t="n">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A6)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A6))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A6)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A6))</f>
         <v>46317</v>
       </c>
     </row>
@@ -3466,19 +3523,19 @@
         <v>108</v>
       </c>
       <c r="C7" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$263,A7)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$264,A7)</f>
         <v>7</v>
       </c>
       <c r="D7" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A7,Plan!$F$5:$F$263,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A7,Plan!$F$5:$F$264,"Done")</f>
         <v>0</v>
       </c>
       <c r="E7" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A7,Plan!$F$5:$F$263,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A7,Plan!$F$5:$F$264,"In progress")</f>
         <v>4</v>
       </c>
       <c r="F7" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A7,Plan!$F$5:$F$263,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A7,Plan!$F$5:$F$264,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G7" s="15" t="n">
@@ -3490,11 +3547,11 @@
         <v>0</v>
       </c>
       <c r="I7" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A7)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A7))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A7)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A7))</f>
         <v>46317</v>
       </c>
       <c r="J7" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A7)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A7))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A7)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A7))</f>
         <v/>
       </c>
     </row>
@@ -3506,19 +3563,19 @@
         <v>137</v>
       </c>
       <c r="C8" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$263,A8)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$264,A8)</f>
         <v>6</v>
       </c>
       <c r="D8" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A8,Plan!$F$5:$F$263,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A8,Plan!$F$5:$F$264,"Done")</f>
         <v>1</v>
       </c>
       <c r="E8" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A8,Plan!$F$5:$F$263,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A8,Plan!$F$5:$F$264,"In progress")</f>
         <v>3</v>
       </c>
       <c r="F8" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A8,Plan!$F$5:$F$263,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A8,Plan!$F$5:$F$264,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G8" s="15" t="n">
@@ -3530,11 +3587,11 @@
         <v>0.166666666666667</v>
       </c>
       <c r="I8" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A8)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A8))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A8)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A8))</f>
         <v>46317</v>
       </c>
       <c r="J8" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A8)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A8))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A8)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A8))</f>
         <v/>
       </c>
     </row>
@@ -3546,19 +3603,19 @@
         <v>161</v>
       </c>
       <c r="C9" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$263,A9)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$264,A9)</f>
         <v>11</v>
       </c>
       <c r="D9" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A9,Plan!$F$5:$F$263,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A9,Plan!$F$5:$F$264,"Done")</f>
         <v>0</v>
       </c>
       <c r="E9" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A9,Plan!$F$5:$F$263,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A9,Plan!$F$5:$F$264,"In progress")</f>
         <v>7</v>
       </c>
       <c r="F9" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A9,Plan!$F$5:$F$263,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A9,Plan!$F$5:$F$264,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G9" s="15" t="n">
@@ -3570,11 +3627,11 @@
         <v>0</v>
       </c>
       <c r="I9" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A9)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A9))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A9)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A9))</f>
         <v>46317</v>
       </c>
       <c r="J9" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A9)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A9))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A9)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A9))</f>
         <v/>
       </c>
     </row>
@@ -3586,19 +3643,19 @@
         <v>202</v>
       </c>
       <c r="C10" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$263,A10)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$264,A10)</f>
         <v>5</v>
       </c>
       <c r="D10" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A10,Plan!$F$5:$F$263,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A10,Plan!$F$5:$F$264,"Done")</f>
         <v>0</v>
       </c>
       <c r="E10" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A10,Plan!$F$5:$F$263,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A10,Plan!$F$5:$F$264,"In progress")</f>
         <v>1</v>
       </c>
       <c r="F10" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A10,Plan!$F$5:$F$263,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A10,Plan!$F$5:$F$264,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G10" s="15" t="n">
@@ -3610,11 +3667,11 @@
         <v>0</v>
       </c>
       <c r="I10" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A10)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A10))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A10)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A10))</f>
         <v>46317</v>
       </c>
       <c r="J10" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A10)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A10))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A10)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A10))</f>
         <v/>
       </c>
     </row>
@@ -3626,20 +3683,20 @@
         <v>219</v>
       </c>
       <c r="C11" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$263,A11)</f>
-        <v>7</v>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$264,A11)</f>
+        <v>8</v>
       </c>
       <c r="D11" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A11,Plan!$F$5:$F$263,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A11,Plan!$F$5:$F$264,"Done")</f>
         <v>0</v>
       </c>
       <c r="E11" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A11,Plan!$F$5:$F$263,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A11,Plan!$F$5:$F$264,"In progress")</f>
         <v>0</v>
       </c>
       <c r="F11" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$263,$A11,Plan!$F$5:$F$263,"Blocked")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A11,Plan!$F$5:$F$264,"Blocked")</f>
+        <v>1</v>
       </c>
       <c r="G11" s="15" t="n">
         <f aca="false">C11-D11-E11-F11</f>
@@ -3650,22 +3707,22 @@
         <v>0</v>
       </c>
       <c r="I11" s="17" t="str">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A11)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$263,Plan!$A$5:$A$263,A11))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A11)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A11))</f>
         <v/>
       </c>
       <c r="J11" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A11)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$263,Plan!$A$5:$A$263,A11))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A11)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A11))</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18"/>
       <c r="B12" s="18" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="C12" s="18" t="n">
         <f aca="false">SUM(C4:C11)</f>
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D12" s="18" t="n">
         <f aca="false">SUM(D4:D11)</f>
@@ -3677,7 +3734,7 @@
       </c>
       <c r="F12" s="18" t="n">
         <f aca="false">SUM(F4:F11)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" s="18" t="n">
         <f aca="false">SUM(G4:G11)</f>
@@ -3685,14 +3742,14 @@
       </c>
       <c r="H12" s="19" t="n">
         <f aca="false">IF(C12=0,0,D12/C12)</f>
-        <v>0.254237288135593</v>
+        <v>0.25</v>
       </c>
       <c r="I12" s="18"/>
       <c r="J12" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>
@@ -3705,7 +3762,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{405640DE-A7CB-41B0-B4DB-6B9D1A6464E3}</x14:id>
+          <x14:id>{9AE83FEA-7481-40F0-8199-52DEC6FA7D96}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3721,7 +3778,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{405640DE-A7CB-41B0-B4DB-6B9D1A6464E3}">
+          <x14:cfRule type="dataBar" id="{9AE83FEA-7481-40F0-8199-52DEC6FA7D96}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
Demo products for testing, new home section types, bulk prices at checkout
- supabase/seed: 100 demo products (one per sub-category) from 3 demo sellers covering new/pre-owned/give-away, free/Featured, sale/flash sale, simple/with options, stock states, pre-order, bulk prices, delivery limits, no COD, a service; demo home sections; remove script
- 0023: home sections for products with options, brand new, price negotiable (home page + admin)
- 0024 + cartlib: bulk prices are used in the cart and when the order is placed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Plan!$A$4:$J$64</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Plan!$A$4:$J$65</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="258">
   <si>
     <t xml:space="preserve">RGBKart Marketplace – Project Plan</t>
   </si>
@@ -787,6 +787,18 @@
   </si>
   <si>
     <t xml:space="preserve">PENDING, set up later (owner, 23 Oct): waits for the real domain. Steps: Resend account + domain DNS records in Hostinger; deploy Edge Function send-alerts (in the repo); secrets RESEND_API_KEY, ALERT_FROM, SITE_URL; Supabase Cron every 5 min; first add a rule so only recent alerts are emailed. Alerts already show on the site (0021_alerts.sql run)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove demo data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delete the 3 demo sellers, their 100 demo products and the demo home sections before launch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run supabase/seed/demo_products_remove.sql in the SQL Editor (added 23 Oct for study and testing)</t>
   </si>
   <si>
     <t xml:space="preserve">Progress by phase</t>
@@ -1426,7 +1438,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -3302,12 +3314,41 @@
         <v>246</v>
       </c>
     </row>
+    <row r="65" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B65" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="C65" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="D65" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="E65" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="F65" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="G65" s="8"/>
+      <c r="H65" s="8"/>
+      <c r="I65" s="14" t="str">
+        <f aca="false">IF(AND(G65&lt;&gt;"",H65&lt;&gt;""),H65-G65+1,"")</f>
+        <v/>
+      </c>
+      <c r="J65" s="10" t="s">
+        <v>250</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J64"/>
+  <autoFilter ref="A4:J65"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F264">
+  <conditionalFormatting sqref="F5:F265">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>$F5="Done"</formula>
     </cfRule>
@@ -3319,11 +3360,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F264" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F265" type="list">
       <formula1>"Not started,In progress,Blocked,Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Enter a date, e.g. 22-Oct-2026" errorStyle="stop" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G5:H264" type="date">
+    <dataValidation allowBlank="true" error="Enter a date, e.g. 22-Oct-2026" errorStyle="stop" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G5:H265" type="date">
       <formula1>DATE(2020,1,1)</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3360,7 +3401,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3371,7 +3412,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>16</v>
@@ -3386,13 +3427,13 @@
         <v>124</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3403,19 +3444,19 @@
         <v>12</v>
       </c>
       <c r="C4" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$264,A4)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$265,A4)</f>
         <v>7</v>
       </c>
       <c r="D4" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A4,Plan!$F$5:$F$264,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A4,Plan!$F$5:$F$265,"Done")</f>
         <v>6</v>
       </c>
       <c r="E4" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A4,Plan!$F$5:$F$264,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A4,Plan!$F$5:$F$265,"In progress")</f>
         <v>1</v>
       </c>
       <c r="F4" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A4,Plan!$F$5:$F$264,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A4,Plan!$F$5:$F$265,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G4" s="15" t="n">
@@ -3427,11 +3468,11 @@
         <v>0.857142857142857</v>
       </c>
       <c r="I4" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A4)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A4))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A4)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A4))</f>
         <v>46317</v>
       </c>
       <c r="J4" s="17" t="n">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A4)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A4))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A4)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A4))</f>
         <v>46317</v>
       </c>
     </row>
@@ -3443,19 +3484,19 @@
         <v>42</v>
       </c>
       <c r="C5" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$264,A5)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$265,A5)</f>
         <v>8</v>
       </c>
       <c r="D5" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A5,Plan!$F$5:$F$264,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A5,Plan!$F$5:$F$265,"Done")</f>
         <v>7</v>
       </c>
       <c r="E5" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A5,Plan!$F$5:$F$264,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A5,Plan!$F$5:$F$265,"In progress")</f>
         <v>1</v>
       </c>
       <c r="F5" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A5,Plan!$F$5:$F$264,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A5,Plan!$F$5:$F$265,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G5" s="15" t="n">
@@ -3467,11 +3508,11 @@
         <v>0.875</v>
       </c>
       <c r="I5" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A5)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A5))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A5)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A5))</f>
         <v>46317</v>
       </c>
       <c r="J5" s="17" t="n">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A5)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A5))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A5)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A5))</f>
         <v>46317</v>
       </c>
     </row>
@@ -3483,19 +3524,19 @@
         <v>75</v>
       </c>
       <c r="C6" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$264,A6)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$265,A6)</f>
         <v>8</v>
       </c>
       <c r="D6" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A6,Plan!$F$5:$F$264,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A6,Plan!$F$5:$F$265,"Done")</f>
         <v>1</v>
       </c>
       <c r="E6" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A6,Plan!$F$5:$F$264,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A6,Plan!$F$5:$F$265,"In progress")</f>
         <v>7</v>
       </c>
       <c r="F6" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A6,Plan!$F$5:$F$264,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A6,Plan!$F$5:$F$265,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G6" s="15" t="n">
@@ -3507,11 +3548,11 @@
         <v>0.125</v>
       </c>
       <c r="I6" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A6)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A6))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A6)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A6))</f>
         <v>46317</v>
       </c>
       <c r="J6" s="17" t="n">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A6)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A6))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A6)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A6))</f>
         <v>46317</v>
       </c>
     </row>
@@ -3523,19 +3564,19 @@
         <v>108</v>
       </c>
       <c r="C7" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$264,A7)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$265,A7)</f>
         <v>7</v>
       </c>
       <c r="D7" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A7,Plan!$F$5:$F$264,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A7,Plan!$F$5:$F$265,"Done")</f>
         <v>0</v>
       </c>
       <c r="E7" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A7,Plan!$F$5:$F$264,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A7,Plan!$F$5:$F$265,"In progress")</f>
         <v>4</v>
       </c>
       <c r="F7" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A7,Plan!$F$5:$F$264,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A7,Plan!$F$5:$F$265,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G7" s="15" t="n">
@@ -3547,11 +3588,11 @@
         <v>0</v>
       </c>
       <c r="I7" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A7)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A7))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A7)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A7))</f>
         <v>46317</v>
       </c>
       <c r="J7" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A7)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A7))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A7)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A7))</f>
         <v/>
       </c>
     </row>
@@ -3563,19 +3604,19 @@
         <v>137</v>
       </c>
       <c r="C8" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$264,A8)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$265,A8)</f>
         <v>6</v>
       </c>
       <c r="D8" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A8,Plan!$F$5:$F$264,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A8,Plan!$F$5:$F$265,"Done")</f>
         <v>1</v>
       </c>
       <c r="E8" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A8,Plan!$F$5:$F$264,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A8,Plan!$F$5:$F$265,"In progress")</f>
         <v>3</v>
       </c>
       <c r="F8" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A8,Plan!$F$5:$F$264,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A8,Plan!$F$5:$F$265,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G8" s="15" t="n">
@@ -3587,11 +3628,11 @@
         <v>0.166666666666667</v>
       </c>
       <c r="I8" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A8)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A8))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A8)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A8))</f>
         <v>46317</v>
       </c>
       <c r="J8" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A8)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A8))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A8)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A8))</f>
         <v/>
       </c>
     </row>
@@ -3603,19 +3644,19 @@
         <v>161</v>
       </c>
       <c r="C9" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$264,A9)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$265,A9)</f>
         <v>11</v>
       </c>
       <c r="D9" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A9,Plan!$F$5:$F$264,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A9,Plan!$F$5:$F$265,"Done")</f>
         <v>0</v>
       </c>
       <c r="E9" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A9,Plan!$F$5:$F$264,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A9,Plan!$F$5:$F$265,"In progress")</f>
         <v>7</v>
       </c>
       <c r="F9" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A9,Plan!$F$5:$F$264,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A9,Plan!$F$5:$F$265,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G9" s="15" t="n">
@@ -3627,11 +3668,11 @@
         <v>0</v>
       </c>
       <c r="I9" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A9)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A9))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A9)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A9))</f>
         <v>46317</v>
       </c>
       <c r="J9" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A9)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A9))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A9)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A9))</f>
         <v/>
       </c>
     </row>
@@ -3643,19 +3684,19 @@
         <v>202</v>
       </c>
       <c r="C10" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$264,A10)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$265,A10)</f>
         <v>5</v>
       </c>
       <c r="D10" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A10,Plan!$F$5:$F$264,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A10,Plan!$F$5:$F$265,"Done")</f>
         <v>0</v>
       </c>
       <c r="E10" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A10,Plan!$F$5:$F$264,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A10,Plan!$F$5:$F$265,"In progress")</f>
         <v>1</v>
       </c>
       <c r="F10" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A10,Plan!$F$5:$F$264,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A10,Plan!$F$5:$F$265,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G10" s="15" t="n">
@@ -3667,11 +3708,11 @@
         <v>0</v>
       </c>
       <c r="I10" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A10)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A10))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A10)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A10))</f>
         <v>46317</v>
       </c>
       <c r="J10" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A10)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A10))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A10)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A10))</f>
         <v/>
       </c>
     </row>
@@ -3683,46 +3724,46 @@
         <v>219</v>
       </c>
       <c r="C11" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$264,A11)</f>
-        <v>8</v>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$265,A11)</f>
+        <v>9</v>
       </c>
       <c r="D11" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A11,Plan!$F$5:$F$264,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A11,Plan!$F$5:$F$265,"Done")</f>
         <v>0</v>
       </c>
       <c r="E11" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A11,Plan!$F$5:$F$264,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A11,Plan!$F$5:$F$265,"In progress")</f>
         <v>0</v>
       </c>
       <c r="F11" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$264,$A11,Plan!$F$5:$F$264,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A11,Plan!$F$5:$F$265,"Blocked")</f>
         <v>1</v>
       </c>
       <c r="G11" s="15" t="n">
         <f aca="false">C11-D11-E11-F11</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H11" s="16" t="n">
         <f aca="false">IF(C11=0,0,D11/C11)</f>
         <v>0</v>
       </c>
       <c r="I11" s="17" t="str">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A11)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$264,Plan!$A$5:$A$264,A11))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A11)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A11))</f>
         <v/>
       </c>
       <c r="J11" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A11)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$264,Plan!$A$5:$A$264,A11))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A11)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A11))</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18"/>
       <c r="B12" s="18" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="C12" s="18" t="n">
         <f aca="false">SUM(C4:C11)</f>
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D12" s="18" t="n">
         <f aca="false">SUM(D4:D11)</f>
@@ -3738,18 +3779,18 @@
       </c>
       <c r="G12" s="18" t="n">
         <f aca="false">SUM(G4:G11)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H12" s="19" t="n">
         <f aca="false">IF(C12=0,0,D12/C12)</f>
-        <v>0.25</v>
+        <v>0.245901639344262</v>
       </c>
       <c r="I12" s="18"/>
       <c r="J12" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>
@@ -3762,7 +3803,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9AE83FEA-7481-40F0-8199-52DEC6FA7D96}</x14:id>
+          <x14:id>{26F16F7C-904C-4C2E-90C5-8E3340D73A64}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3778,7 +3819,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9AE83FEA-7481-40F0-8199-52DEC6FA7D96}">
+          <x14:cfRule type="dataBar" id="{26F16F7C-904C-4C2E-90C5-8E3340D73A64}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
Seller shop page (store.html)
- Public page per shop: banner, logo, name, tagline, location, since, product count, pickup, call / WhatsApp / email, social links, holiday notice, about
- Shop's products with search, category buttons, sort, 20 per page with Previous / Next
- Links from product page (Visit shop), cart and My orders; English / Bangla
- Page-number styles moved to shop.css; plan row 1.8 done

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -270,7 +270,7 @@
     <t xml:space="preserve">Public page per shop: logo, banner, products</t>
   </si>
   <si>
-    <t xml:space="preserve">Shop settings built 22 Oct (shop_settings.sql): logo, banner, web address, contact, social links, vacation mode, payout details. Public shop page still to build</t>
+    <t xml:space="preserve">Shop settings built 22 Oct (shop_settings.sql): logo, banner, web address, contact, social links, vacation mode, payout details. Public shop page still to build · 23 Oct: store.html?s=&lt;shop&gt; with banner, logo, contact, about, search, category filter, sort and pages; linked from product, cart and orders</t>
   </si>
   <si>
     <t xml:space="preserve">Customer Shopping</t>
@@ -1960,7 +1960,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="n">
         <v>1</v>
       </c>
@@ -1977,15 +1977,17 @@
         <v>73</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="G19" s="8" t="n">
         <v>46317</v>
       </c>
-      <c r="H19" s="8"/>
-      <c r="I19" s="14" t="str">
+      <c r="H19" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I19" s="14" t="n">
         <f aca="false">IF(AND(G19&lt;&gt;"",H19&lt;&gt;""),H19-G19+1,"")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J19" s="10" t="s">
         <v>74</v>
@@ -3489,11 +3491,11 @@
       </c>
       <c r="D5" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A5,Plan!$F$5:$F$265,"Done")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E5" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A5,Plan!$F$5:$F$265,"In progress")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" s="15" t="n">
         <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A5,Plan!$F$5:$F$265,"Blocked")</f>
@@ -3505,7 +3507,7 @@
       </c>
       <c r="H5" s="16" t="n">
         <f aca="false">IF(C5=0,0,D5/C5)</f>
-        <v>0.875</v>
+        <v>1</v>
       </c>
       <c r="I5" s="17" t="n">
         <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A5)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A5))</f>
@@ -3767,11 +3769,11 @@
       </c>
       <c r="D12" s="18" t="n">
         <f aca="false">SUM(D4:D11)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E12" s="18" t="n">
         <f aca="false">SUM(E4:E11)</f>
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F12" s="18" t="n">
         <f aca="false">SUM(F4:F11)</f>
@@ -3783,7 +3785,7 @@
       </c>
       <c r="H12" s="19" t="n">
         <f aca="false">IF(C12=0,0,D12/C12)</f>
-        <v>0.245901639344262</v>
+        <v>0.262295081967213</v>
       </c>
       <c r="I12" s="18"/>
       <c r="J12" s="18"/>
@@ -3803,7 +3805,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{26F16F7C-904C-4C2E-90C5-8E3340D73A64}</x14:id>
+          <x14:id>{4CB15574-88C7-4FCC-9590-E5D48FBD8810}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3819,7 +3821,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{26F16F7C-904C-4C2E-90C5-8E3340D73A64}">
+          <x14:cfRule type="dataBar" id="{4CB15574-88C7-4FCC-9590-E5D48FBD8810}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
Plan: 3.1 done; new phase 8 lists extra work done on request; notes on 2.1, 2.2, 5.1-5.3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Plan!$A$4:$J$65</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Plan!$A$4:$J$82</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="322">
   <si>
     <t xml:space="preserve">RGBKart Marketplace – Project Plan</t>
   </si>
@@ -285,7 +285,7 @@
     <t xml:space="preserve">Banners, featured categories, new and popular products</t>
   </si>
   <si>
-    <t xml:space="preserve">Updated 22 Oct: 6×2 category cards, All categories page (categories.html), admin-managed product sections (Featured, Deals of the Day, New arrivals…), New/Pre-owned/Sale labels, heart, cart icon with count. Banners editable later (5.9)</t>
+    <t xml:space="preserve">Updated 22 Oct: 6×2 category cards, All categories page (categories.html), admin-managed product sections (Featured, Deals of the Day, New arrivals…), New/Pre-owned/Sale labels, heart, cart icon with count. Banners editable later (5.9) · 23 Oct: Top shops sliding row, new section types (with options, brand new, negotiable), category pictures</t>
   </si>
   <si>
     <t xml:space="preserve">2.2</t>
@@ -297,7 +297,7 @@
     <t xml:space="preserve">Browse by category; filter by price, brand, rating; sort</t>
   </si>
   <si>
-    <t xml:space="preserve">Built 22 Oct (browse.html): left sidebar with expandable categories, filters (condition, price, district, featured, free delivery), sort, show more</t>
+    <t xml:space="preserve">Built 22 Oct (browse.html): left sidebar with expandable categories, filters (condition, price, district, featured, free delivery), sort, show more · 23 Oct: page numbers with Previous / Next (24 per page), fixed header and menu, coloured sub-category buttons, picture icons in the sidebar</t>
   </si>
   <si>
     <t xml:space="preserve">2.3</t>
@@ -384,7 +384,7 @@
     <t xml:space="preserve">Customers save delivery addresses (division, district, area)</t>
   </si>
   <si>
-    <t xml:space="preserve">Checkout remembers the last address on the device and fills it from the customer profile; full address book later</t>
+    <t xml:space="preserve">Checkout remembers the last address on the device and fills it from the customer profile; full address book later · 23 Oct: account.html (profile, tiles, saved addresses up to 10 with a default, recent orders, change password); checkout picks a saved address and can save a new one (0028_customer_account.sql)</t>
   </si>
   <si>
     <t xml:space="preserve">3.2</t>
@@ -543,6 +543,9 @@
     <t xml:space="preserve">Platform commission per category or seller</t>
   </si>
   <si>
+    <t xml:space="preserve">Probably not needed: owner rule is zero commission and sellers collect cash on delivery themselves. Confirm before building</t>
+  </si>
+  <si>
     <t xml:space="preserve">5.2</t>
   </si>
   <si>
@@ -799,6 +802,195 @@
   </si>
   <si>
     <t xml:space="preserve">Run supabase/seed/demo_products_remove.sql in the SQL Editor (added 23 Oct for study and testing)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extra work (added on owner's request)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brand header &amp; logo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basket logo with 'Red &amp; Green Basket' wordmark in logo colours on a white pill; green band with yellow rule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 Oct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Password eye &amp; confirm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show/hide password on every password box; confirm password on sign-up and reset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Main menu editor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin → Main menu: links, hot items, groups of categories (Electronics, Fashion)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 Oct (0016, 0017)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-time seller Free / Featured</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sell.html: free listing (message only, phone hidden) or Featured (call, WhatsApp, email); enforced in the database</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin tools</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin adds products (RGBKart Official or a seller), gives Featured free, sets ad rates, books ads, reports with CSV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 Oct (0018)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payments check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bKash, Nagad, Upay, Rocket numbers; one TrxID can be used only once; admin verifies and Featured / ad starts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 Oct (0019)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alerts page &amp; bell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alerts page, bell in header with unread count, email on/off switch (emails wait for 7.8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 Oct (0021)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Language switch with flags</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bangladesh / UK flag button in menu bar, footer, sign-in and sell pages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 Oct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demo data for testing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 demo products (every case), 12 demo shops, demo home sections; remove before launch (7.9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 Oct (supabase/seed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed header &amp; menu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Header and main menu stay at the top while scrolling on every shop page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page numbers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Previous / Next and page numbers on product lists and shop pages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pictures by admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upload a picture per category; add, remove and re-order photos of any product</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 Oct (0025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shop page look</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Picture icons in the category sidebar, light green sidebar, brand-coloured sub-category buttons</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visit shop button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Green 'Visit shop' button on the product page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Top shops sliding row</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home page row of shops (logo, banner, name, counts), glides continuously; admin sets movement, speed, direction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 Oct (0026, 0027)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">More home section types</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sections for products with options, brand new only, price negotiable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 Oct (0023)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulk prices at checkout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Buy more, pay less' prices now charged in the cart and the order (was only shown)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 Oct (0024)</t>
   </si>
   <si>
     <t xml:space="preserve">Progress by phase</t>
@@ -1438,7 +1630,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:J82"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -1993,7 +2185,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="n">
         <v>2</v>
       </c>
@@ -2024,7 +2216,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="n">
         <v>2</v>
       </c>
@@ -2243,7 +2435,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="n">
         <v>3</v>
       </c>
@@ -2260,15 +2452,17 @@
         <v>111</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H28" s="8"/>
-      <c r="I28" s="14" t="str">
+        <v>46318</v>
+      </c>
+      <c r="H28" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I28" s="14" t="n">
         <f aca="false">IF(AND(G28&lt;&gt;"",H28&lt;&gt;""),H28-G28+1,"")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J28" s="10" t="s">
         <v>112</v>
@@ -2632,7 +2826,7 @@
       </c>
       <c r="J40" s="10"/>
     </row>
-    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="n">
         <v>5</v>
       </c>
@@ -2657,9 +2851,11 @@
         <f aca="false">IF(AND(G41&lt;&gt;"",H41&lt;&gt;""),H41-G41+1,"")</f>
         <v/>
       </c>
-      <c r="J41" s="10"/>
-    </row>
-    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J41" s="10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="n">
         <v>5</v>
       </c>
@@ -2667,13 +2863,13 @@
         <v>161</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F42" s="7" t="s">
         <v>124</v>
@@ -2684,9 +2880,11 @@
         <f aca="false">IF(AND(G42&lt;&gt;"",H42&lt;&gt;""),H42-G42+1,"")</f>
         <v/>
       </c>
-      <c r="J42" s="10"/>
-    </row>
-    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J42" s="10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="n">
         <v>5</v>
       </c>
@@ -2694,13 +2892,13 @@
         <v>161</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F43" s="7" t="s">
         <v>124</v>
@@ -2711,7 +2909,9 @@
         <f aca="false">IF(AND(G43&lt;&gt;"",H43&lt;&gt;""),H43-G43+1,"")</f>
         <v/>
       </c>
-      <c r="J43" s="10"/>
+      <c r="J43" s="10" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="11" t="n">
@@ -2721,13 +2921,13 @@
         <v>161</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D44" s="12" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E44" s="12" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F44" s="7" t="s">
         <v>28</v>
@@ -2741,7 +2941,7 @@
         <v/>
       </c>
       <c r="J44" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2752,13 +2952,13 @@
         <v>161</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D45" s="12" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E45" s="12" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F45" s="7" t="s">
         <v>28</v>
@@ -2772,7 +2972,7 @@
         <v/>
       </c>
       <c r="J45" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2783,13 +2983,13 @@
         <v>161</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D46" s="12" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E46" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F46" s="7" t="s">
         <v>28</v>
@@ -2803,7 +3003,7 @@
         <v/>
       </c>
       <c r="J46" s="10" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2814,13 +3014,13 @@
         <v>161</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E47" s="12" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F47" s="7" t="s">
         <v>28</v>
@@ -2834,7 +3034,7 @@
         <v/>
       </c>
       <c r="J47" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2845,13 +3045,13 @@
         <v>161</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D48" s="12" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E48" s="12" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F48" s="7" t="s">
         <v>28</v>
@@ -2865,7 +3065,7 @@
         <v/>
       </c>
       <c r="J48" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2876,13 +3076,13 @@
         <v>161</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D49" s="12" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E49" s="12" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F49" s="7" t="s">
         <v>28</v>
@@ -2896,7 +3096,7 @@
         <v/>
       </c>
       <c r="J49" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2907,13 +3107,13 @@
         <v>161</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F50" s="7" t="s">
         <v>28</v>
@@ -2927,7 +3127,7 @@
         <v/>
       </c>
       <c r="J50" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2938,13 +3138,13 @@
         <v>161</v>
       </c>
       <c r="C51" s="13" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D51" s="12" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E51" s="12" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F51" s="7" t="s">
         <v>124</v>
@@ -2962,16 +3162,16 @@
         <v>6</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F52" s="7" t="s">
         <v>124</v>
@@ -2989,16 +3189,16 @@
         <v>6</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F53" s="7" t="s">
         <v>28</v>
@@ -3012,7 +3212,7 @@
         <v/>
       </c>
       <c r="J53" s="10" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3020,16 +3220,16 @@
         <v>6</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F54" s="7" t="s">
         <v>124</v>
@@ -3047,16 +3247,16 @@
         <v>6</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F55" s="7" t="s">
         <v>124</v>
@@ -3074,16 +3274,16 @@
         <v>6</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F56" s="7" t="s">
         <v>124</v>
@@ -3101,16 +3301,16 @@
         <v>7</v>
       </c>
       <c r="B57" s="12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F57" s="7" t="s">
         <v>124</v>
@@ -3128,16 +3328,16 @@
         <v>7</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D58" s="12" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E58" s="12" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F58" s="7" t="s">
         <v>124</v>
@@ -3149,7 +3349,7 @@
         <v/>
       </c>
       <c r="J58" s="10" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3157,16 +3357,16 @@
         <v>7</v>
       </c>
       <c r="B59" s="12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E59" s="12" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F59" s="7" t="s">
         <v>124</v>
@@ -3184,16 +3384,16 @@
         <v>7</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D60" s="12" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E60" s="12" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F60" s="7" t="s">
         <v>124</v>
@@ -3211,16 +3411,16 @@
         <v>7</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C61" s="13" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E61" s="12" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F61" s="7" t="s">
         <v>124</v>
@@ -3238,16 +3438,16 @@
         <v>7</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D62" s="12" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E62" s="12" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F62" s="7" t="s">
         <v>124</v>
@@ -3265,16 +3465,16 @@
         <v>7</v>
       </c>
       <c r="B63" s="12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C63" s="13" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D63" s="12" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E63" s="12" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F63" s="7" t="s">
         <v>124</v>
@@ -3292,19 +3492,19 @@
         <v>7</v>
       </c>
       <c r="B64" s="12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C64" s="13" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D64" s="12" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E64" s="12" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F64" s="7" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="G64" s="8"/>
       <c r="H64" s="8"/>
@@ -3313,7 +3513,7 @@
         <v/>
       </c>
       <c r="J64" s="10" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3321,16 +3521,16 @@
         <v>7</v>
       </c>
       <c r="B65" s="12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C65" s="13" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D65" s="12" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E65" s="12" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F65" s="7" t="s">
         <v>124</v>
@@ -3342,15 +3542,576 @@
         <v/>
       </c>
       <c r="J65" s="10" t="s">
-        <v>250</v>
+        <v>251</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B66" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="D66" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="E66" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="F66" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G66" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H66" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I66" s="9" t="n">
+        <f aca="false">IF(AND(G66&lt;&gt;"",H66&lt;&gt;""),H66-G66+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J66" s="10" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B67" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="D67" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="E67" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="F67" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G67" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H67" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I67" s="9" t="n">
+        <f aca="false">IF(AND(G67&lt;&gt;"",H67&lt;&gt;""),H67-G67+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J67" s="10" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="D68" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="E68" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="F68" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G68" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H68" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I68" s="9" t="n">
+        <f aca="false">IF(AND(G68&lt;&gt;"",H68&lt;&gt;""),H68-G68+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J68" s="10" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B69" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="D69" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F69" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G69" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H69" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I69" s="9" t="n">
+        <f aca="false">IF(AND(G69&lt;&gt;"",H69&lt;&gt;""),H69-G69+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J69" s="10" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B70" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="D70" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="F70" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G70" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H70" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I70" s="9" t="n">
+        <f aca="false">IF(AND(G70&lt;&gt;"",H70&lt;&gt;""),H70-G70+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J70" s="10" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B71" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="D71" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="F71" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G71" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H71" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I71" s="9" t="n">
+        <f aca="false">IF(AND(G71&lt;&gt;"",H71&lt;&gt;""),H71-G71+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J71" s="10" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B72" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="D72" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="F72" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G72" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H72" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I72" s="9" t="n">
+        <f aca="false">IF(AND(G72&lt;&gt;"",H72&lt;&gt;""),H72-G72+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J72" s="10" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B73" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="D73" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="E73" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="F73" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G73" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H73" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I73" s="9" t="n">
+        <f aca="false">IF(AND(G73&lt;&gt;"",H73&lt;&gt;""),H73-G73+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J73" s="10" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B74" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="F74" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G74" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H74" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I74" s="9" t="n">
+        <f aca="false">IF(AND(G74&lt;&gt;"",H74&lt;&gt;""),H74-G74+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J74" s="10" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B75" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="E75" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="F75" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G75" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H75" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I75" s="9" t="n">
+        <f aca="false">IF(AND(G75&lt;&gt;"",H75&lt;&gt;""),H75-G75+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J75" s="10" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B76" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="D76" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="E76" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="F76" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G76" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H76" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I76" s="9" t="n">
+        <f aca="false">IF(AND(G76&lt;&gt;"",H76&lt;&gt;""),H76-G76+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J76" s="10" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B77" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="D77" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="E77" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="F77" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G77" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H77" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I77" s="9" t="n">
+        <f aca="false">IF(AND(G77&lt;&gt;"",H77&lt;&gt;""),H77-G77+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J77" s="10" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B78" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="D78" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="E78" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="F78" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G78" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H78" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I78" s="9" t="n">
+        <f aca="false">IF(AND(G78&lt;&gt;"",H78&lt;&gt;""),H78-G78+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J78" s="10" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B79" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="D79" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="E79" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="F79" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G79" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H79" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I79" s="9" t="n">
+        <f aca="false">IF(AND(G79&lt;&gt;"",H79&lt;&gt;""),H79-G79+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J79" s="10" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B80" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="D80" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="E80" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="F80" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G80" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H80" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I80" s="9" t="n">
+        <f aca="false">IF(AND(G80&lt;&gt;"",H80&lt;&gt;""),H80-G80+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J80" s="10" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B81" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="D81" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="E81" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="F81" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G81" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H81" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I81" s="9" t="n">
+        <f aca="false">IF(AND(G81&lt;&gt;"",H81&lt;&gt;""),H81-G81+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J81" s="10" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B82" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="D82" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="E82" s="5" t="s">
+        <v>313</v>
+      </c>
+      <c r="F82" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G82" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H82" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I82" s="9" t="n">
+        <f aca="false">IF(AND(G82&lt;&gt;"",H82&lt;&gt;""),H82-G82+1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="J82" s="10" t="s">
+        <v>314</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J65"/>
+  <autoFilter ref="A4:J82"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F265">
+  <conditionalFormatting sqref="F5:F282">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>$F5="Done"</formula>
     </cfRule>
@@ -3362,11 +4123,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F265" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F282" type="list">
       <formula1>"Not started,In progress,Blocked,Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Enter a date, e.g. 22-Oct-2026" errorStyle="stop" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G5:H265" type="date">
+    <dataValidation allowBlank="true" error="Enter a date, e.g. 22-Oct-2026" errorStyle="stop" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G5:H282" type="date">
       <formula1>DATE(2020,1,1)</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3388,7 +4149,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -3403,7 +4164,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>251</v>
+        <v>315</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3414,7 +4175,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>252</v>
+        <v>316</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>16</v>
@@ -3423,19 +4184,19 @@
         <v>28</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>124</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>253</v>
+        <v>317</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>254</v>
+        <v>318</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>255</v>
+        <v>319</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3446,19 +4207,19 @@
         <v>12</v>
       </c>
       <c r="C4" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$265,A4)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$282,A4)</f>
         <v>7</v>
       </c>
       <c r="D4" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A4,Plan!$F$5:$F$265,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A4,Plan!$F$5:$F$282,"Done")</f>
         <v>6</v>
       </c>
       <c r="E4" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A4,Plan!$F$5:$F$265,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A4,Plan!$F$5:$F$282,"In progress")</f>
         <v>1</v>
       </c>
       <c r="F4" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A4,Plan!$F$5:$F$265,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A4,Plan!$F$5:$F$282,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G4" s="15" t="n">
@@ -3470,11 +4231,11 @@
         <v>0.857142857142857</v>
       </c>
       <c r="I4" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A4)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A4))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A4)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A4))</f>
         <v>46317</v>
       </c>
       <c r="J4" s="17" t="n">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A4)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A4))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A4)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A4))</f>
         <v>46317</v>
       </c>
     </row>
@@ -3486,19 +4247,19 @@
         <v>42</v>
       </c>
       <c r="C5" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$265,A5)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$282,A5)</f>
         <v>8</v>
       </c>
       <c r="D5" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A5,Plan!$F$5:$F$265,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A5,Plan!$F$5:$F$282,"Done")</f>
         <v>8</v>
       </c>
       <c r="E5" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A5,Plan!$F$5:$F$265,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A5,Plan!$F$5:$F$282,"In progress")</f>
         <v>0</v>
       </c>
       <c r="F5" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A5,Plan!$F$5:$F$265,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A5,Plan!$F$5:$F$282,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G5" s="15" t="n">
@@ -3510,11 +4271,11 @@
         <v>1</v>
       </c>
       <c r="I5" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A5)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A5))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A5)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A5))</f>
         <v>46317</v>
       </c>
       <c r="J5" s="17" t="n">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A5)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A5))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A5)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A5))</f>
         <v>46317</v>
       </c>
     </row>
@@ -3526,19 +4287,19 @@
         <v>75</v>
       </c>
       <c r="C6" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$265,A6)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$282,A6)</f>
         <v>8</v>
       </c>
       <c r="D6" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A6,Plan!$F$5:$F$265,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A6,Plan!$F$5:$F$282,"Done")</f>
         <v>1</v>
       </c>
       <c r="E6" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A6,Plan!$F$5:$F$265,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A6,Plan!$F$5:$F$282,"In progress")</f>
         <v>7</v>
       </c>
       <c r="F6" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A6,Plan!$F$5:$F$265,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A6,Plan!$F$5:$F$282,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G6" s="15" t="n">
@@ -3550,11 +4311,11 @@
         <v>0.125</v>
       </c>
       <c r="I6" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A6)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A6))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A6)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A6))</f>
         <v>46317</v>
       </c>
       <c r="J6" s="17" t="n">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A6)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A6))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A6)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A6))</f>
         <v>46317</v>
       </c>
     </row>
@@ -3566,19 +4327,19 @@
         <v>108</v>
       </c>
       <c r="C7" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$265,A7)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$282,A7)</f>
         <v>7</v>
       </c>
       <c r="D7" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A7,Plan!$F$5:$F$265,"Done")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A7,Plan!$F$5:$F$282,"Done")</f>
+        <v>1</v>
       </c>
       <c r="E7" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A7,Plan!$F$5:$F$265,"In progress")</f>
-        <v>4</v>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A7,Plan!$F$5:$F$282,"In progress")</f>
+        <v>3</v>
       </c>
       <c r="F7" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A7,Plan!$F$5:$F$265,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A7,Plan!$F$5:$F$282,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G7" s="15" t="n">
@@ -3587,15 +4348,15 @@
       </c>
       <c r="H7" s="16" t="n">
         <f aca="false">IF(C7=0,0,D7/C7)</f>
-        <v>0</v>
+        <v>0.142857142857143</v>
       </c>
       <c r="I7" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A7)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A7))</f>
-        <v>46317</v>
-      </c>
-      <c r="J7" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A7)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A7))</f>
-        <v/>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A7)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A7))</f>
+        <v>46317</v>
+      </c>
+      <c r="J7" s="17" t="n">
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A7)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A7))</f>
+        <v>46318</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3606,19 +4367,19 @@
         <v>137</v>
       </c>
       <c r="C8" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$265,A8)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$282,A8)</f>
         <v>6</v>
       </c>
       <c r="D8" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A8,Plan!$F$5:$F$265,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A8,Plan!$F$5:$F$282,"Done")</f>
         <v>1</v>
       </c>
       <c r="E8" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A8,Plan!$F$5:$F$265,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A8,Plan!$F$5:$F$282,"In progress")</f>
         <v>3</v>
       </c>
       <c r="F8" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A8,Plan!$F$5:$F$265,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A8,Plan!$F$5:$F$282,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G8" s="15" t="n">
@@ -3630,11 +4391,11 @@
         <v>0.166666666666667</v>
       </c>
       <c r="I8" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A8)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A8))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A8)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A8))</f>
         <v>46317</v>
       </c>
       <c r="J8" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A8)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A8))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A8)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A8))</f>
         <v/>
       </c>
     </row>
@@ -3646,19 +4407,19 @@
         <v>161</v>
       </c>
       <c r="C9" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$265,A9)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$282,A9)</f>
         <v>11</v>
       </c>
       <c r="D9" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A9,Plan!$F$5:$F$265,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A9,Plan!$F$5:$F$282,"Done")</f>
         <v>0</v>
       </c>
       <c r="E9" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A9,Plan!$F$5:$F$265,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A9,Plan!$F$5:$F$282,"In progress")</f>
         <v>7</v>
       </c>
       <c r="F9" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A9,Plan!$F$5:$F$265,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A9,Plan!$F$5:$F$282,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G9" s="15" t="n">
@@ -3670,11 +4431,11 @@
         <v>0</v>
       </c>
       <c r="I9" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A9)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A9))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A9)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A9))</f>
         <v>46317</v>
       </c>
       <c r="J9" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A9)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A9))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A9)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A9))</f>
         <v/>
       </c>
     </row>
@@ -3683,22 +4444,22 @@
         <v>6</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C10" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$265,A10)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$282,A10)</f>
         <v>5</v>
       </c>
       <c r="D10" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A10,Plan!$F$5:$F$265,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A10,Plan!$F$5:$F$282,"Done")</f>
         <v>0</v>
       </c>
       <c r="E10" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A10,Plan!$F$5:$F$265,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A10,Plan!$F$5:$F$282,"In progress")</f>
         <v>1</v>
       </c>
       <c r="F10" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A10,Plan!$F$5:$F$265,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A10,Plan!$F$5:$F$282,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G10" s="15" t="n">
@@ -3710,11 +4471,11 @@
         <v>0</v>
       </c>
       <c r="I10" s="17" t="n">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A10)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A10))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A10)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A10))</f>
         <v>46317</v>
       </c>
       <c r="J10" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A10)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A10))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A10)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A10))</f>
         <v/>
       </c>
     </row>
@@ -3723,22 +4484,22 @@
         <v>7</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C11" s="15" t="n">
-        <f aca="false">COUNTIF(Plan!$A$5:$A$265,A11)</f>
+        <f aca="false">COUNTIF(Plan!$A$5:$A$282,A11)</f>
         <v>9</v>
       </c>
       <c r="D11" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A11,Plan!$F$5:$F$265,"Done")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A11,Plan!$F$5:$F$282,"Done")</f>
         <v>0</v>
       </c>
       <c r="E11" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A11,Plan!$F$5:$F$265,"In progress")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A11,Plan!$F$5:$F$282,"In progress")</f>
         <v>0</v>
       </c>
       <c r="F11" s="15" t="n">
-        <f aca="false">COUNTIFS(Plan!$A$5:$A$265,$A11,Plan!$F$5:$F$265,"Blocked")</f>
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A11,Plan!$F$5:$F$282,"Blocked")</f>
         <v>1</v>
       </c>
       <c r="G11" s="15" t="n">
@@ -3750,53 +4511,93 @@
         <v>0</v>
       </c>
       <c r="I11" s="17" t="str">
-        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A11)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$265,Plan!$A$5:$A$265,A11))</f>
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A11)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A11))</f>
         <v/>
       </c>
       <c r="J11" s="17" t="str">
-        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A11)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$265,Plan!$A$5:$A$265,A11))</f>
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A11)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A11))</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18"/>
-      <c r="B12" s="18" t="s">
-        <v>256</v>
-      </c>
-      <c r="C12" s="18" t="n">
-        <f aca="false">SUM(C4:C11)</f>
-        <v>61</v>
-      </c>
-      <c r="D12" s="18" t="n">
-        <f aca="false">SUM(D4:D11)</f>
-        <v>16</v>
-      </c>
-      <c r="E12" s="18" t="n">
-        <f aca="false">SUM(E4:E11)</f>
-        <v>23</v>
-      </c>
-      <c r="F12" s="18" t="n">
-        <f aca="false">SUM(F4:F11)</f>
-        <v>1</v>
-      </c>
-      <c r="G12" s="18" t="n">
-        <f aca="false">SUM(G4:G11)</f>
+      <c r="A12" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>252</v>
+      </c>
+      <c r="C12" s="15" t="n">
+        <f aca="false">COUNTIF(Plan!$A$5:$A$282,A12)</f>
+        <v>17</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A12,Plan!$F$5:$F$282,"Done")</f>
+        <v>17</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A12,Plan!$F$5:$F$282,"In progress")</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="15" t="n">
+        <f aca="false">COUNTIFS(Plan!$A$5:$A$282,$A12,Plan!$F$5:$F$282,"Blocked")</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="15" t="n">
+        <f aca="false">C12-D12-E12-F12</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="16" t="n">
+        <f aca="false">IF(C12=0,0,D12/C12)</f>
+        <v>1</v>
+      </c>
+      <c r="I12" s="17" t="n">
+        <f aca="false">IF(_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A12)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$282,Plan!$A$5:$A$282,A12))</f>
+        <v>46317</v>
+      </c>
+      <c r="J12" s="17" t="n">
+        <f aca="false">IF(_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A12)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$282,Plan!$A$5:$A$282,A12))</f>
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18"/>
+      <c r="B13" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="C13" s="18" t="n">
+        <f aca="false">SUM(C4:C12)</f>
+        <v>78</v>
+      </c>
+      <c r="D13" s="18" t="n">
+        <f aca="false">SUM(D4:D12)</f>
+        <v>34</v>
+      </c>
+      <c r="E13" s="18" t="n">
+        <f aca="false">SUM(E4:E12)</f>
+        <v>22</v>
+      </c>
+      <c r="F13" s="18" t="n">
+        <f aca="false">SUM(F4:F12)</f>
+        <v>1</v>
+      </c>
+      <c r="G13" s="18" t="n">
+        <f aca="false">SUM(G4:G12)</f>
         <v>21</v>
       </c>
-      <c r="H12" s="19" t="n">
-        <f aca="false">IF(C12=0,0,D12/C12)</f>
-        <v>0.262295081967213</v>
-      </c>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
-        <v>257</v>
+      <c r="H13" s="19" t="n">
+        <f aca="false">IF(C13=0,0,D13/C13)</f>
+        <v>0.435897435897436</v>
+      </c>
+      <c r="I13" s="18"/>
+      <c r="J13" s="18"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="20" t="s">
+        <v>321</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H4:H12">
+  <conditionalFormatting sqref="H4:H13">
     <cfRule type="dataBar" priority="2">
       <dataBar showValue="1" minLength="10" maxLength="90">
         <cfvo type="num" val="0"/>
@@ -3805,7 +4606,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4CB15574-88C7-4FCC-9590-E5D48FBD8810}</x14:id>
+          <x14:id>{6019F119-13C3-49B0-A473-C060BC5BEBB0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3821,7 +4622,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4CB15574-88C7-4FCC-9590-E5D48FBD8810}">
+          <x14:cfRule type="dataBar" id="{6019F119-13C3-49B0-A473-C060BC5BEBB0}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -3833,7 +4634,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>H4:H12</xm:sqref>
+          <xm:sqref>H4:H13</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
Reviews & ratings (plan 6.1): buyers rate shop and products after delivery, stars on cards/product/shop pages, seller replies, admin hide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -2689,16 +2689,24 @@
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G52" s="8" t="n"/>
-      <c r="H52" s="8" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G52" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H52" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I52" s="9">
         <f>IF(AND(G52&lt;&gt;"",H52&lt;&gt;""),H52-G52+1,"")</f>
         <v/>
       </c>
-      <c r="J52" s="10" t="inlineStr"/>
+      <c r="J52" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct (0029_reviews.sql): after delivery the buyer rates the shop and each product (stars + comment) on My orders; stars on product cards, product page, shop page and Top shops; Top rated sort and 4-star filter; shop replies in Seller Center → Reviews; staff hide/show in Admin → Reviews. Demo reviews: supabase/seed/demo_reviews.sql</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">

</xml_diff>

<commit_message>
Fraud & reports (plan 6.5): report product/shop, Admin → Complaints, risky COD buyer check in Seller Center; plan 5.1–5.3 not needed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -146,7 +146,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -183,6 +183,19 @@
         <patternFill patternType="solid">
           <fgColor rgb="00F8E3E0"/>
           <bgColor rgb="00F8E3E0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="0078858F"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00ECEFF1"/>
+          <bgColor rgb="00ECEFF1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2228,7 +2241,7 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Not needed</t>
         </is>
       </c>
       <c r="G41" s="8" t="n"/>
@@ -2239,7 +2252,7 @@
       </c>
       <c r="J41" s="10" t="inlineStr">
         <is>
-          <t>Probably not needed: owner rule is zero commission and sellers collect cash on delivery themselves. Confirm before building</t>
+          <t>Not needed (owner, 23 Oct): zero commission, and sellers collect cash on delivery themselves, so RGBKart holds no seller money. Payouts button removed from Seller Center.</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2282,7 @@
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Not needed</t>
         </is>
       </c>
       <c r="G42" s="8" t="n"/>
@@ -2280,7 +2293,7 @@
       </c>
       <c r="J42" s="10" t="inlineStr">
         <is>
-          <t>Probably not needed: owner rule is zero commission and sellers collect cash on delivery themselves. Confirm before building</t>
+          <t>Not needed (owner, 23 Oct): zero commission, and sellers collect cash on delivery themselves, so RGBKart holds no seller money. Payouts button removed from Seller Center.</t>
         </is>
       </c>
     </row>
@@ -2310,7 +2323,7 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Not needed</t>
         </is>
       </c>
       <c r="G43" s="8" t="n"/>
@@ -2321,7 +2334,7 @@
       </c>
       <c r="J43" s="10" t="inlineStr">
         <is>
-          <t>Probably not needed: owner rule is zero commission and sellers collect cash on delivery themselves. Confirm before building</t>
+          <t>Not needed (owner, 23 Oct): zero commission, and sellers collect cash on delivery themselves, so RGBKart holds no seller money. Payouts button removed from Seller Center.</t>
         </is>
       </c>
     </row>
@@ -2851,16 +2864,24 @@
       </c>
       <c r="F56" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G56" s="8" t="n"/>
-      <c r="H56" s="8" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G56" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H56" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I56" s="9">
         <f>IF(AND(G56&lt;&gt;"",H56&lt;&gt;""),H56-G56+1,"")</f>
         <v/>
       </c>
-      <c r="J56" s="10" t="inlineStr"/>
+      <c r="J56" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct (0030_reports_fraud.sql): Report this product / shop on product, shop and My orders pages (also guests); Admin → Complaints (to check / closed, note, resolved / dismissed, reporter alerted); Seller Center orders show buyer history from all shops (delivered, refused, cancelled) with Risky / Check first / Trusted / New labels; quick cancel reasons incl. Customer refused the parcel</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
@@ -4032,10 +4053,13 @@
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>$F5="Blocked"</formula>
     </cfRule>
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>$F5="Not needed"</formula>
+    </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation sqref="F5:F283" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Not started,In progress,Blocked,Done"</formula1>
+      <formula1>"Not started,In progress,Blocked,Done,Not needed"</formula1>
     </dataValidation>
     <dataValidation sqref="G5:H283" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Enter a date, e.g. 22-Oct-2026" type="date" operator="greaterThan">
       <formula1>DATE(2020,1,1)</formula1>
@@ -4136,7 +4160,7 @@
         </is>
       </c>
       <c r="C4" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A4)</f>
+        <f>COUNTIF(Plan!$A$5:$A$283,A4)-COUNTIFS(Plan!$A$5:$A$283,A4,Plan!$F$5:$F$283,"Not needed")</f>
         <v/>
       </c>
       <c r="D4" s="15">
@@ -4178,7 +4202,7 @@
         </is>
       </c>
       <c r="C5" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A5)</f>
+        <f>COUNTIF(Plan!$A$5:$A$283,A5)-COUNTIFS(Plan!$A$5:$A$283,A5,Plan!$F$5:$F$283,"Not needed")</f>
         <v/>
       </c>
       <c r="D5" s="15">
@@ -4220,7 +4244,7 @@
         </is>
       </c>
       <c r="C6" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A6)</f>
+        <f>COUNTIF(Plan!$A$5:$A$283,A6)-COUNTIFS(Plan!$A$5:$A$283,A6,Plan!$F$5:$F$283,"Not needed")</f>
         <v/>
       </c>
       <c r="D6" s="15">
@@ -4262,7 +4286,7 @@
         </is>
       </c>
       <c r="C7" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A7)</f>
+        <f>COUNTIF(Plan!$A$5:$A$283,A7)-COUNTIFS(Plan!$A$5:$A$283,A7,Plan!$F$5:$F$283,"Not needed")</f>
         <v/>
       </c>
       <c r="D7" s="15">
@@ -4304,7 +4328,7 @@
         </is>
       </c>
       <c r="C8" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A8)</f>
+        <f>COUNTIF(Plan!$A$5:$A$283,A8)-COUNTIFS(Plan!$A$5:$A$283,A8,Plan!$F$5:$F$283,"Not needed")</f>
         <v/>
       </c>
       <c r="D8" s="15">
@@ -4346,7 +4370,7 @@
         </is>
       </c>
       <c r="C9" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A9)</f>
+        <f>COUNTIF(Plan!$A$5:$A$283,A9)-COUNTIFS(Plan!$A$5:$A$283,A9,Plan!$F$5:$F$283,"Not needed")</f>
         <v/>
       </c>
       <c r="D9" s="15">
@@ -4388,7 +4412,7 @@
         </is>
       </c>
       <c r="C10" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A10)</f>
+        <f>COUNTIF(Plan!$A$5:$A$283,A10)-COUNTIFS(Plan!$A$5:$A$283,A10,Plan!$F$5:$F$283,"Not needed")</f>
         <v/>
       </c>
       <c r="D10" s="15">
@@ -4430,7 +4454,7 @@
         </is>
       </c>
       <c r="C11" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A11)</f>
+        <f>COUNTIF(Plan!$A$5:$A$283,A11)-COUNTIFS(Plan!$A$5:$A$283,A11,Plan!$F$5:$F$283,"Not needed")</f>
         <v/>
       </c>
       <c r="D11" s="15">
@@ -4472,7 +4496,7 @@
         </is>
       </c>
       <c r="C12" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A12)</f>
+        <f>COUNTIF(Plan!$A$5:$A$283,A12)-COUNTIFS(Plan!$A$5:$A$283,A12,Plan!$F$5:$F$283,"Not needed")</f>
         <v/>
       </c>
       <c r="D12" s="15">
@@ -4541,7 +4565,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Counts and dates come from the Plan tab. Status values: Not started, In progress, Blocked, Done.</t>
+          <t>Counts and dates come from the Plan tab. Status values: Not started, In progress, Blocked, Done, Not needed (left out of the counts).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wishlist & cart in the customer account (plan 2.5/2.6): sync across devices, merge at sign-in, clear at sign-out
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -1524,20 +1524,22 @@
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G24" s="8" t="n">
         <v>46317</v>
       </c>
-      <c r="H24" s="8" t="n"/>
+      <c r="H24" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I24" s="9">
         <f>IF(AND(G24&lt;&gt;"",H24&lt;&gt;""),H24-G24+1,"")</f>
         <v/>
       </c>
       <c r="J24" s="10" t="inlineStr">
         <is>
-          <t>Heart on every product card; saved on the device for now. Moves to the account when customer accounts are finished</t>
+          <t>23 Oct (0031_saved_lists.sql): saved items kept in the customer account (customer_lists) and on every device; merged at sign-in, cleared from the device at sign-out</t>
         </is>
       </c>
     </row>
@@ -1567,20 +1569,22 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G25" s="8" t="n">
         <v>46317</v>
       </c>
-      <c r="H25" s="8" t="n"/>
+      <c r="H25" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I25" s="9">
         <f>IF(AND(G25&lt;&gt;"",H25&lt;&gt;""),H25-G25+1,"")</f>
         <v/>
       </c>
       <c r="J25" s="10" t="inlineStr">
         <is>
-          <t>23 Oct: cart grouped by shop with live prices/stock and delivery choice; saved on the device (moves to the account later)</t>
+          <t>23 Oct (0031_saved_lists.sql): cart kept in the customer account and on every device (sync.js); prices/stock still checked live and by place_order</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Product Q&A (plan 6.3): ask on product page, seller answers (page or Seller Center), alerts, admin hide; free listings can't share contact in answers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -2794,16 +2794,24 @@
       </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G54" s="8" t="n"/>
-      <c r="H54" s="8" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G54" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H54" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I54" s="9">
         <f>IF(AND(G54&lt;&gt;"",H54&lt;&gt;""),H54-G54+1,"")</f>
         <v/>
       </c>
-      <c r="J54" s="10" t="inlineStr"/>
+      <c r="J54" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct (0032_product_questions.sql): Questions &amp; answers on product pages (guests too); seller answers on the product page or Seller Center → Questions; buyer alerted; free one-time listings cannot put phone/email/links in answers; Admin → Questions hide/show</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n">

</xml_diff>

<commit_message>
Shop coupons (plan 3.6): Seller Center → Coupons, coupon box per shop in cart, checked again in place_order; discount on invoices and orders
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -1910,21 +1910,29 @@
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>Admin-created discount codes</t>
+          <t>Shop discount codes</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G33" s="8" t="n"/>
-      <c r="H33" s="8" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H33" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I33" s="14">
         <f>IF(AND(G33&lt;&gt;"",H33&lt;&gt;""),H33-G33+1,"")</f>
         <v/>
       </c>
-      <c r="J33" s="10" t="inlineStr"/>
+      <c r="J33" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct (0033_shop_coupons.sql): each shop makes its own codes in Seller Center → Coupons (taka or % off, cap, minimum order, dates, total and per-buyer limits, on/off); buyers apply them per shop in the cart; place_order checks again, records the use, total = items + delivery − discount; cancelled orders give the use back; shown on invoices and My orders. Zero commission: the shop gives the discount</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="n">

</xml_diff>

<commit_message>
Returns (plan 4.6): customers request returns after delivery within return days, shops accept/decline/receive (stock back), admin overview, private photos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -2216,16 +2216,24 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G40" s="8" t="n"/>
-      <c r="H40" s="8" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H40" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I40" s="9">
         <f>IF(AND(G40&lt;&gt;"",H40&lt;&gt;""),H40-G40+1,"")</f>
         <v/>
       </c>
-      <c r="J40" s="10" t="inlineStr"/>
+      <c r="J40" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct (0036_returns.sql): My orders → Return this item within the product's return days (saved on the order line); reason, refund or exchange, details, up to 3 private photos; shop accepts / declines / marks item received (stock back) in Seller Center → Returns; admin sees all in Admin → Returns; alerts both ways. Refund paid by the shop directly (RGBKart holds no money)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="11" t="n">

</xml_diff>

<commit_message>
Admin activity log (plan 5.11): staff changes recorded by the database, Admin → Activity log with filters and CSV
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -2685,16 +2685,24 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G51" s="8" t="n"/>
-      <c r="H51" s="8" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G51" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H51" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I51" s="14">
         <f>IF(AND(G51&lt;&gt;"",H51&lt;&gt;""),H51-G51+1,"")</f>
         <v/>
       </c>
-      <c r="J51" s="10" t="inlineStr"/>
+      <c r="J51" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct (0037_activity_log.sql): database triggers on 26 tables record every add/change/delete made by staff (who, role, when, what changed from → to); Admin → Activity log for Master Admin and Co-admins with filters, search and CSV download; entries cannot be edited or deleted</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n">

</xml_diff>

<commit_message>
Seller verification (plan 6.4): shops send NID/trade licence privately, admin approves, Verified shop badge for buyers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -2863,16 +2863,24 @@
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G55" s="8" t="n"/>
-      <c r="H55" s="8" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G55" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H55" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I55" s="9">
         <f>IF(AND(G55&lt;&gt;"",H55&lt;&gt;""),H55-G55+1,"")</f>
         <v/>
       </c>
-      <c r="J55" s="10" t="inlineStr"/>
+      <c r="J55" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct (0038_seller_verification.sql): Seller Center → Get verified (NID / trade licence / passport, up to 4 private files); Admin → Verification approve / reject with note, remove badge; '✓ Verified shop' on shop page, product page and Top shops; only staff can set the badge</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n">

</xml_diff>

<commit_message>
Policy pages (plan 7.3): About, Contact, Terms, Privacy, Returns, Seller rules in English and Bangla, footer links, Admin → Pages & policies editor
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -3031,16 +3031,22 @@
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G59" s="8" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="G59" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="H59" s="8" t="n"/>
       <c r="I59" s="14">
         <f>IF(AND(G59&lt;&gt;"",H59&lt;&gt;""),H59-G59+1,"")</f>
         <v/>
       </c>
-      <c r="J59" s="10" t="inlineStr"/>
+      <c r="J59" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct (0039_site_pages.sql): About, Contact, Terms, Privacy, Return &amp; refund, Seller rules pages in English and Bangla (page.html?p=…), linked in every footer, editable in Admin → Pages &amp; policies. TO DO by owner: fill the [square bracket] parts (support email/phone, address, date) and have a lawyer check Terms and Privacy</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">

</xml_diff>

<commit_message>
Search engines & speed (plan 7.6): page tags, link previews (share.php + Share button), Google product details, nightly sitemap, robots, 404, caching/compression, app manifest
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -3148,16 +3148,24 @@
       </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G62" s="8" t="n"/>
-      <c r="H62" s="8" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G62" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H62" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I62" s="14">
         <f>IF(AND(G62&lt;&gt;"",H62&lt;&gt;""),H62-G62+1,"")</f>
         <v/>
       </c>
-      <c r="J62" s="10" t="inlineStr"/>
+      <c r="J62" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct: page descriptions and share tags on every page, branded share picture, share.php link previews for products and shops (Facebook / WhatsApp / Messenger) + Share button, Google product details (price, stock, stars), sitemap.xml rebuilt every night by the deploy workflow, robots.txt (private pages hidden), 404 page, .htaccess compression and caching, app manifest. Set repository variable SITE_URL when the real domain is ready</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">

</xml_diff>

<commit_message>
Security review (plan 7.4): read-only public views, Featured lock enforced, safer uploads and default rights; report in docs/SECURITY_REVIEW.md
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -3074,16 +3074,22 @@
       </c>
       <c r="F60" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G60" s="8" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="G60" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="H60" s="8" t="n"/>
       <c r="I60" s="14">
         <f>IF(AND(G60&lt;&gt;"",H60&lt;&gt;""),H60-G60+1,"")</f>
         <v/>
       </c>
-      <c r="J60" s="10" t="inlineStr"/>
+      <c r="J60" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct: review done (docs/SECURITY_REVIEW.md). 0040_security_fixes.sql fixes public reviews/questions being editable by anyone, enforces the Featured lock, tightens return-photo uploads and default rights. Owner to do: run 0040, Supabase Security Advisor screenshot, CAPTCHA + backups before launch</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">

</xml_diff>

<commit_message>
Cash on Delivery limits (plan 3.3): per-shop order cap, first-order cap, orders on the way per buyer
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -1794,7 +1794,7 @@
         </is>
       </c>
       <c r="G30" s="8" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="H30" s="8" t="n"/>
       <c r="I30" s="14">
@@ -1803,7 +1803,7 @@
       </c>
       <c r="J30" s="10" t="inlineStr">
         <is>
-          <t>Cash on Delivery is the only payment; RGBKart never holds money. Order limits per day in place</t>
+          <t>23 Oct: COD limits (0041_cod_limits.sql): biggest order per shop, lower first-order limit, orders on the way per buyer; set in Admin → Orders; checked by the database; checkout warns. Done once 0041 is run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
COD limits box: tidy layout; 0041 run on live
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -1790,20 +1790,22 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G30" s="8" t="n">
         <v>46318</v>
       </c>
-      <c r="H30" s="8" t="n"/>
+      <c r="H30" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I30" s="14">
         <f>IF(AND(G30&lt;&gt;"",H30&lt;&gt;""),H30-G30+1,"")</f>
         <v/>
       </c>
       <c r="J30" s="10" t="inlineStr">
         <is>
-          <t>23 Oct: COD limits (0041_cod_limits.sql): biggest order per shop, lower first-order limit, orders on the way per buyer; set in Admin → Orders; checked by the database; checkout warns. Done once 0041 is run</t>
+          <t>23 Oct: COD limits (0041_cod_limits.sql): biggest order per shop, lower first-order limit, orders on the way per buyer; set in Admin → Orders; checked by the database; checkout warns. 0041 run 23 Oct</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Search (plan 2.3): match every word across product, category and shop; Shops row; Featured first then newest
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -1438,20 +1438,22 @@
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G22" s="8" t="n">
         <v>46317</v>
       </c>
-      <c r="H22" s="8" t="n"/>
+      <c r="H22" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I22" s="9">
         <f>IF(AND(G22&lt;&gt;"",H22&lt;&gt;""),H22-G22+1,"")</f>
         <v/>
       </c>
       <c r="J22" s="10" t="inlineStr">
         <is>
-          <t>Built 22 Oct: search by name, description and tags; matching categories suggested. Cart page (cart.html) added</t>
+          <t>23 Oct: every word must match the product (name, description, code, tag), its category or its shop; matching shops shown in a row above the results, matching categories as buttons; results Featured first, then newest published; English and Bangla</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports (plan 5.10): top shops and products, full Excel download (built-in xlsx writer)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -2177,20 +2177,22 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G39" s="8" t="n">
         <v>46317</v>
       </c>
-      <c r="H39" s="8" t="n"/>
+      <c r="H39" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I39" s="9">
         <f>IF(AND(G39&lt;&gt;"",H39&lt;&gt;""),H39-G39+1,"")</f>
         <v/>
       </c>
       <c r="J39" s="10" t="inlineStr">
         <is>
-          <t>23 Oct: 0042_cancel_rules.sql: admin sets until which step buyers cancel themselves (New/Confirmed/Packed) and whether a reason is required; after that buyers ask the shop to cancel, shop accepts or declines with a note; alerts both ways; shops always give a reason. Done once 0042 is run</t>
+          <t>23 Oct: 0042_cancel_rules.sql: admin sets until which step buyers cancel themselves (New/Confirmed/Packed) and whether a reason is required; after that buyers ask the shop to cancel, shop accepts or declines with a note; alerts both ways; shops always give a reason. 0042 run 23 Oct</t>
         </is>
       </c>
     </row>
@@ -2646,20 +2648,22 @@
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G50" s="8" t="n">
         <v>46317</v>
       </c>
-      <c r="H50" s="8" t="n"/>
+      <c r="H50" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I50" s="14">
         <f>IF(AND(G50&lt;&gt;"",H50&lt;&gt;""),H50-G50+1,"")</f>
         <v/>
       </c>
       <c r="J50" s="10" t="inlineStr">
         <is>
-          <t>23 Oct: Admin → Reports: daily/weekly/monthly/yearly/custom; visitors, sign-ups, listings, Featured &amp; ad income; charts; CSV download. Sales/orders come with checkout</t>
+          <t>23 Oct: Admin → Reports adds Top shops and Top products for any period; Download Excel = one workbook (Summary, Orders, Payments received, Top shops, Top products) made by site/xlsx-lite.js, no outside library; CSV summary kept</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Demo data removed on live (sections kept); plan 7.9 done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -3285,18 +3285,22 @@
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G65" s="8" t="n"/>
-      <c r="H65" s="8" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G65" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H65" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I65" s="14">
         <f>IF(AND(G65&lt;&gt;"",H65&lt;&gt;""),H65-G65+1,"")</f>
         <v/>
       </c>
       <c r="J65" s="10" t="inlineStr">
         <is>
-          <t>Run supabase/seed/demo_products_remove.sql in the SQL Editor (added 23 Oct for study and testing)</t>
+          <t>23 Oct: all demo shops, products, buyers, orders and reviews removed (demo_remove_keep_sections.sql); the 14 home page sections were kept by the owner's choice</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Project plan updated (domain move, email, testing, new rows 8.19–8.23)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan'!$A$4:$J$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan'!$A$4:$J$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -576,7 +576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -962,7 +962,7 @@
       </c>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>All 3 SQL files run OK; hkmanik@gmail.com is Master Admin (22 Oct). To do: URL Configuration, open admin.html, test sign-in flows</t>
+          <t>All 3 SQL files run OK. 23 Oct: Master Admin moved to rgbkart@gmail.com (0046); hkmanik@gmail.com is now a Co-admin</t>
         </is>
       </c>
     </row>
@@ -2956,21 +2956,27 @@
       </c>
       <c r="E57" s="12" t="inlineStr">
         <is>
-          <t>Put site online (e.g. Vercel/Netlify) on your domain</t>
+          <t>Put the site online on Hostinger on your own domain (rgbkart.com)</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G57" s="8" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="G57" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="H57" s="8" t="n"/>
       <c r="I57" s="14">
         <f>IF(AND(G57&lt;&gt;"",H57&lt;&gt;""),H57-G57+1,"")</f>
         <v/>
       </c>
-      <c r="J57" s="10" t="inlineStr"/>
+      <c r="J57" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct: rgbkart.com renewed (active until 14 Aug 2027, auto-renewal on). Old WordPress site on rgbkart.com deleted (mailboxes kept). Next: empty PHP/HTML website on rgbkart.com → FTP login → GitHub secrets + SITE_URL=https://rgbkart.com → Supabase allowed addresses → forward rgbkartdemo.hkmanik.com and www to rgbkart.com</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
@@ -3009,7 +3015,7 @@
       </c>
       <c r="J58" s="10" t="inlineStr">
         <is>
-          <t>Supabase free email is limited to a few per hour</t>
+          <t>Do together with 7.8 after the domain: Resend (account under rgbkart@gmail.com) as Supabase's email sender, so sign-up / password emails are not limited (23 Oct the built-in sender hit its hourly limit)</t>
         </is>
       </c>
     </row>
@@ -3125,16 +3131,22 @@
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G61" s="8" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="G61" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="H61" s="8" t="n"/>
       <c r="I61" s="14">
         <f>IF(AND(G61&lt;&gt;"",H61&lt;&gt;""),H61-G61+1,"")</f>
         <v/>
       </c>
-      <c r="J61" s="10" t="inlineStr"/>
+      <c r="J61" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct: owner's full check as buyer, shop and admin started; demo data removed, so test with real test shops and products</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
@@ -3255,7 +3267,7 @@
       </c>
       <c r="J64" s="10" t="inlineStr">
         <is>
-          <t>PENDING, set up later (owner, 23 Oct): waits for the real domain. Steps: Resend account + domain DNS records in Hostinger; deploy Edge Function send-alerts (in the repo); secrets RESEND_API_KEY, ALERT_FROM, SITE_URL; Supabase Cron every 5 min; first add a rule so only recent alerts are emailed. Alerts already show on the site (0021_alerts.sql run)</t>
+          <t>Waits for 7.1 (rgbkart.com live). Then: Resend account under rgbkart@gmail.com, verify rgbkart.com in Hostinger DNS, send from alerts@rgbkart.com; Edge Function send-alerts + Cron every 5 min; only recent alerts emailed (old ones skipped)</t>
         </is>
       </c>
     </row>
@@ -4114,12 +4126,237 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Extra work (added on owner's request)</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>8.19</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>VAT on invoices</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>Admin switches VAT on/off, default rate, VAT per category and per product; VAT shown per item on invoices and orders</t>
+        </is>
+      </c>
+      <c r="F84" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G84" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H84" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I84" s="9">
+        <f>IF(AND(G84&lt;&gt;"",H84&lt;&gt;""),H84-G84+1,"")</f>
+        <v/>
+      </c>
+      <c r="J84" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct (0043, 0044): VAT off until the owner switches it on in Admin → Orders</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Extra work (added on owner's request)</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>8.20</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>Delivery set by each shop</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>Admin delivery methods with suggested and maximum fees, special methods for heavy, vehicle, flammable, fragile; each shop ticks methods, sets fees and free delivery above an amount</t>
+        </is>
+      </c>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G85" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H85" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I85" s="9">
+        <f>IF(AND(G85&lt;&gt;"",H85&lt;&gt;""),H85-G85+1,"")</f>
+        <v/>
+      </c>
+      <c r="J85" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct (0045): Seller Center → Delivery, Admin → Orders → Delivery methods</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Extra work (added on owner's request)</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr">
+        <is>
+          <t>8.21</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>Master Admin account</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>Master Admin moved to rgbkart@gmail.com; hkmanik@gmail.com stays as Co-admin</t>
+        </is>
+      </c>
+      <c r="F86" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G86" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H86" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I86" s="9">
+        <f>IF(AND(G86&lt;&gt;"",H86&lt;&gt;""),H86-G86+1,"")</f>
+        <v/>
+      </c>
+      <c r="J86" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct (0046)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Extra work (added on owner's request)</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>8.22</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>Admin dashboard button</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>'⚙ Admin dashboard' on My account for team members; 'Seller Center' for shops</t>
+        </is>
+      </c>
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G87" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H87" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I87" s="9">
+        <f>IF(AND(G87&lt;&gt;"",H87&lt;&gt;""),H87-G87+1,"")</f>
+        <v/>
+      </c>
+      <c r="J87" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Extra work (added on owner's request)</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="inlineStr">
+        <is>
+          <t>8.23</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>Excel reports without outside tools</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>Download Excel built into the site (xlsx-lite.js); top shops and top products in Reports</t>
+        </is>
+      </c>
+      <c r="F88" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G88" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H88" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I88" s="9">
+        <f>IF(AND(G88&lt;&gt;"",H88&lt;&gt;""),H88-G88+1,"")</f>
+        <v/>
+      </c>
+      <c r="J88" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct (see 5.10)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J83"/>
+  <autoFilter ref="A4:J88"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F283">
+  <conditionalFormatting sqref="F5:F288">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$F5="Done"</formula>
     </cfRule>
@@ -4134,10 +4371,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F283" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F288" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Blocked,Done,Not needed"</formula1>
     </dataValidation>
-    <dataValidation sqref="G5:H283" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Enter a date, e.g. 22-Oct-2026" type="date" operator="greaterThan">
+    <dataValidation sqref="G5:H288" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Enter a date, e.g. 22-Oct-2026" type="date" operator="greaterThan">
       <formula1>DATE(2020,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -4236,19 +4473,19 @@
         </is>
       </c>
       <c r="C4" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A4)-COUNTIFS(Plan!$A$5:$A$283,A4,Plan!$F$5:$F$283,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$288,A4)-COUNTIFS(Plan!$A$5:$A$288,A4,Plan!$F$5:$F$288,"Not needed")</f>
         <v/>
       </c>
       <c r="D4" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A4,Plan!$F$5:$F$283,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A4,Plan!$F$5:$F$288,"Done")</f>
         <v/>
       </c>
       <c r="E4" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A4,Plan!$F$5:$F$283,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A4,Plan!$F$5:$F$288,"In progress")</f>
         <v/>
       </c>
       <c r="F4" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A4,Plan!$F$5:$F$283,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A4,Plan!$F$5:$F$288,"Blocked")</f>
         <v/>
       </c>
       <c r="G4" s="15">
@@ -4260,11 +4497,11 @@
         <v/>
       </c>
       <c r="I4" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A4)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A4))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A4)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A4))</f>
         <v/>
       </c>
       <c r="J4" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A4)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A4))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A4)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A4))</f>
         <v/>
       </c>
     </row>
@@ -4278,19 +4515,19 @@
         </is>
       </c>
       <c r="C5" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A5)-COUNTIFS(Plan!$A$5:$A$283,A5,Plan!$F$5:$F$283,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$288,A5)-COUNTIFS(Plan!$A$5:$A$288,A5,Plan!$F$5:$F$288,"Not needed")</f>
         <v/>
       </c>
       <c r="D5" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A5,Plan!$F$5:$F$283,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A5,Plan!$F$5:$F$288,"Done")</f>
         <v/>
       </c>
       <c r="E5" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A5,Plan!$F$5:$F$283,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A5,Plan!$F$5:$F$288,"In progress")</f>
         <v/>
       </c>
       <c r="F5" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A5,Plan!$F$5:$F$283,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A5,Plan!$F$5:$F$288,"Blocked")</f>
         <v/>
       </c>
       <c r="G5" s="15">
@@ -4302,11 +4539,11 @@
         <v/>
       </c>
       <c r="I5" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A5)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A5))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A5)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A5))</f>
         <v/>
       </c>
       <c r="J5" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A5)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A5))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A5)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A5))</f>
         <v/>
       </c>
     </row>
@@ -4320,19 +4557,19 @@
         </is>
       </c>
       <c r="C6" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A6)-COUNTIFS(Plan!$A$5:$A$283,A6,Plan!$F$5:$F$283,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$288,A6)-COUNTIFS(Plan!$A$5:$A$288,A6,Plan!$F$5:$F$288,"Not needed")</f>
         <v/>
       </c>
       <c r="D6" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A6,Plan!$F$5:$F$283,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A6,Plan!$F$5:$F$288,"Done")</f>
         <v/>
       </c>
       <c r="E6" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A6,Plan!$F$5:$F$283,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A6,Plan!$F$5:$F$288,"In progress")</f>
         <v/>
       </c>
       <c r="F6" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A6,Plan!$F$5:$F$283,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A6,Plan!$F$5:$F$288,"Blocked")</f>
         <v/>
       </c>
       <c r="G6" s="15">
@@ -4344,11 +4581,11 @@
         <v/>
       </c>
       <c r="I6" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A6)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A6))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A6)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A6))</f>
         <v/>
       </c>
       <c r="J6" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A6)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A6))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A6)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A6))</f>
         <v/>
       </c>
     </row>
@@ -4362,19 +4599,19 @@
         </is>
       </c>
       <c r="C7" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A7)-COUNTIFS(Plan!$A$5:$A$283,A7,Plan!$F$5:$F$283,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$288,A7)-COUNTIFS(Plan!$A$5:$A$288,A7,Plan!$F$5:$F$288,"Not needed")</f>
         <v/>
       </c>
       <c r="D7" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A7,Plan!$F$5:$F$283,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A7,Plan!$F$5:$F$288,"Done")</f>
         <v/>
       </c>
       <c r="E7" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A7,Plan!$F$5:$F$283,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A7,Plan!$F$5:$F$288,"In progress")</f>
         <v/>
       </c>
       <c r="F7" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A7,Plan!$F$5:$F$283,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A7,Plan!$F$5:$F$288,"Blocked")</f>
         <v/>
       </c>
       <c r="G7" s="15">
@@ -4386,11 +4623,11 @@
         <v/>
       </c>
       <c r="I7" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A7)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A7))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A7)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A7))</f>
         <v/>
       </c>
       <c r="J7" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A7)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A7))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A7)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A7))</f>
         <v/>
       </c>
     </row>
@@ -4404,19 +4641,19 @@
         </is>
       </c>
       <c r="C8" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A8)-COUNTIFS(Plan!$A$5:$A$283,A8,Plan!$F$5:$F$283,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$288,A8)-COUNTIFS(Plan!$A$5:$A$288,A8,Plan!$F$5:$F$288,"Not needed")</f>
         <v/>
       </c>
       <c r="D8" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A8,Plan!$F$5:$F$283,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A8,Plan!$F$5:$F$288,"Done")</f>
         <v/>
       </c>
       <c r="E8" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A8,Plan!$F$5:$F$283,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A8,Plan!$F$5:$F$288,"In progress")</f>
         <v/>
       </c>
       <c r="F8" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A8,Plan!$F$5:$F$283,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A8,Plan!$F$5:$F$288,"Blocked")</f>
         <v/>
       </c>
       <c r="G8" s="15">
@@ -4428,11 +4665,11 @@
         <v/>
       </c>
       <c r="I8" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A8)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A8))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A8)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A8))</f>
         <v/>
       </c>
       <c r="J8" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A8)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A8))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A8)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A8))</f>
         <v/>
       </c>
     </row>
@@ -4446,19 +4683,19 @@
         </is>
       </c>
       <c r="C9" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A9)-COUNTIFS(Plan!$A$5:$A$283,A9,Plan!$F$5:$F$283,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$288,A9)-COUNTIFS(Plan!$A$5:$A$288,A9,Plan!$F$5:$F$288,"Not needed")</f>
         <v/>
       </c>
       <c r="D9" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A9,Plan!$F$5:$F$283,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A9,Plan!$F$5:$F$288,"Done")</f>
         <v/>
       </c>
       <c r="E9" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A9,Plan!$F$5:$F$283,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A9,Plan!$F$5:$F$288,"In progress")</f>
         <v/>
       </c>
       <c r="F9" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A9,Plan!$F$5:$F$283,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A9,Plan!$F$5:$F$288,"Blocked")</f>
         <v/>
       </c>
       <c r="G9" s="15">
@@ -4470,11 +4707,11 @@
         <v/>
       </c>
       <c r="I9" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A9)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A9))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A9)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A9))</f>
         <v/>
       </c>
       <c r="J9" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A9)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A9))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A9)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A9))</f>
         <v/>
       </c>
     </row>
@@ -4488,19 +4725,19 @@
         </is>
       </c>
       <c r="C10" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A10)-COUNTIFS(Plan!$A$5:$A$283,A10,Plan!$F$5:$F$283,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$288,A10)-COUNTIFS(Plan!$A$5:$A$288,A10,Plan!$F$5:$F$288,"Not needed")</f>
         <v/>
       </c>
       <c r="D10" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A10,Plan!$F$5:$F$283,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A10,Plan!$F$5:$F$288,"Done")</f>
         <v/>
       </c>
       <c r="E10" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A10,Plan!$F$5:$F$283,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A10,Plan!$F$5:$F$288,"In progress")</f>
         <v/>
       </c>
       <c r="F10" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A10,Plan!$F$5:$F$283,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A10,Plan!$F$5:$F$288,"Blocked")</f>
         <v/>
       </c>
       <c r="G10" s="15">
@@ -4512,11 +4749,11 @@
         <v/>
       </c>
       <c r="I10" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A10)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A10))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A10)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A10))</f>
         <v/>
       </c>
       <c r="J10" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A10)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A10))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A10)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A10))</f>
         <v/>
       </c>
     </row>
@@ -4530,19 +4767,19 @@
         </is>
       </c>
       <c r="C11" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A11)-COUNTIFS(Plan!$A$5:$A$283,A11,Plan!$F$5:$F$283,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$288,A11)-COUNTIFS(Plan!$A$5:$A$288,A11,Plan!$F$5:$F$288,"Not needed")</f>
         <v/>
       </c>
       <c r="D11" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A11,Plan!$F$5:$F$283,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A11,Plan!$F$5:$F$288,"Done")</f>
         <v/>
       </c>
       <c r="E11" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A11,Plan!$F$5:$F$283,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A11,Plan!$F$5:$F$288,"In progress")</f>
         <v/>
       </c>
       <c r="F11" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A11,Plan!$F$5:$F$283,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A11,Plan!$F$5:$F$288,"Blocked")</f>
         <v/>
       </c>
       <c r="G11" s="15">
@@ -4554,11 +4791,11 @@
         <v/>
       </c>
       <c r="I11" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A11)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A11))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A11)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A11))</f>
         <v/>
       </c>
       <c r="J11" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A11)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A11))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A11)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A11))</f>
         <v/>
       </c>
     </row>
@@ -4572,19 +4809,19 @@
         </is>
       </c>
       <c r="C12" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$283,A12)-COUNTIFS(Plan!$A$5:$A$283,A12,Plan!$F$5:$F$283,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$288,A12)-COUNTIFS(Plan!$A$5:$A$288,A12,Plan!$F$5:$F$288,"Not needed")</f>
         <v/>
       </c>
       <c r="D12" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A12,Plan!$F$5:$F$283,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A12,Plan!$F$5:$F$288,"Done")</f>
         <v/>
       </c>
       <c r="E12" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A12,Plan!$F$5:$F$283,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A12,Plan!$F$5:$F$288,"In progress")</f>
         <v/>
       </c>
       <c r="F12" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$283,$A12,Plan!$F$5:$F$283,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$288,$A12,Plan!$F$5:$F$288,"Blocked")</f>
         <v/>
       </c>
       <c r="G12" s="15">
@@ -4596,11 +4833,11 @@
         <v/>
       </c>
       <c r="I12" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A12)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$283,Plan!$A$5:$A$283,A12))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A12)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A12))</f>
         <v/>
       </c>
       <c r="J12" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A12)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$283,Plan!$A$5:$A$283,A12))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A12)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A12))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Domain move done: rgbkart.com live, demo forwards; plan 7.1 done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -2961,20 +2961,22 @@
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G57" s="8" t="n">
         <v>46318</v>
       </c>
-      <c r="H57" s="8" t="n"/>
+      <c r="H57" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I57" s="14">
         <f>IF(AND(G57&lt;&gt;"",H57&lt;&gt;""),H57-G57+1,"")</f>
         <v/>
       </c>
       <c r="J57" s="10" t="inlineStr">
         <is>
-          <t>23 Oct: rgbkart.com renewed (active until 14 Aug 2027, auto-renewal on). Old WordPress site on rgbkart.com deleted (mailboxes kept). Next: empty PHP/HTML website on rgbkart.com → FTP login → GitHub secrets + SITE_URL=https://rgbkart.com → Supabase allowed addresses → forward rgbkartdemo.hkmanik.com and www to rgbkart.com</t>
+          <t>23 Oct: live at https://rgbkart.com (renewed to 14 Aug 2027, auto-renewal on). Old WordPress removed (mailboxes kept); new PHP/HTML website with SSL; GitHub uploads there (FTP u456241157.deploy, SITE_URL); Supabase Site URL updated; rgbkartdemo.hkmanik.com forwards to rgbkart.com; www forwards to rgbkart.com</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Email alerts live (0048 run): notes and project plan 6.2, 7.2, 7.8 done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -2783,20 +2783,22 @@
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G53" s="8" t="n">
         <v>46317</v>
       </c>
-      <c r="H53" s="8" t="n"/>
+      <c r="H53" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I53" s="9">
         <f>IF(AND(G53&lt;&gt;"",H53&lt;&gt;""),H53-G53+1,"")</f>
         <v/>
       </c>
       <c r="J53" s="10" t="inlineStr">
         <is>
-          <t>23 Oct: Alerts page + header bell + email via Resend for orders, payments, listing review, shop approval, messages, Featured/ad ending soon. Each person can switch emails off. Email sending pending, see 7.8. SMS later</t>
+          <t>23 Oct: Alerts page + header bell + email via Resend for orders, payments, listing review, shop approval, messages, Featured/ad ending soon. Each person can switch emails off. Emails live 23 Oct (7.8). SMS later</t>
         </is>
       </c>
     </row>
@@ -3006,18 +3008,22 @@
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G58" s="8" t="n"/>
-      <c r="H58" s="8" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G58" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H58" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I58" s="14">
         <f>IF(AND(G58&lt;&gt;"",H58&lt;&gt;""),H58-G58+1,"")</f>
         <v/>
       </c>
       <c r="J58" s="10" t="inlineStr">
         <is>
-          <t>Do together with 7.8 after the domain: Resend (account under rgbkart@gmail.com) as Supabase's email sender, so sign-up / password emails are not limited (23 Oct the built-in sender hit its hourly limit)</t>
+          <t>23 Oct: Supabase Auth sends through Resend SMTP (no-reply@rgbkart.com, 100/hour). Was: do together with 7.8 after the domain: Resend (account under rgbkart@gmail.com) as Supabase's email sender, so sign-up / password emails are not limited (23 Oct the built-in sender hit its hourly limit)</t>
         </is>
       </c>
     </row>
@@ -3258,18 +3264,22 @@
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-      <c r="G64" s="8" t="n"/>
-      <c r="H64" s="8" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G64" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H64" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="I64" s="14">
         <f>IF(AND(G64&lt;&gt;"",H64&lt;&gt;""),H64-G64+1,"")</f>
         <v/>
       </c>
       <c r="J64" s="10" t="inlineStr">
         <is>
-          <t>Waits for 7.1 (rgbkart.com live). Then: Resend account under rgbkart@gmail.com, verify rgbkart.com in Hostinger DNS, send from alerts@rgbkart.com; Edge Function send-alerts + Cron every 5 min; only recent alerts emailed (old ones skipped)</t>
+          <t>23 Oct (0048): test email received. Set up: Resend account under rgbkart@gmail.com, verify rgbkart.com in Hostinger DNS, send from alerts@rgbkart.com; Edge Function send-alerts + Cron every 5 min; only recent alerts emailed (old ones skipped)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Project plan rows 8.24-8.27 and live-site walk-through checklist
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012oyp35F86nsbVYsw11ojW4
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan'!$A$4:$J$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan'!$A$4:$J$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -576,7 +576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4363,12 +4363,190 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>Extra work (added on owner's request)</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="inlineStr">
+        <is>
+          <t>8.24</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>Users page with Block / Delete</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>Admin → Users: every account (staff, shop, one-time seller, customer, guest) with counts; Block / Unblock (Master or Co-admin), Delete permanently (Master only, type the email)</t>
+        </is>
+      </c>
+      <c r="F89" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G89" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H89" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I89" s="9">
+        <f>IF(AND(G89&lt;&gt;"",H89&lt;&gt;""),H89-G89+1,"")</f>
+        <v/>
+      </c>
+      <c r="J89" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct (0047)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Extra work (added on owner's request)</t>
+        </is>
+      </c>
+      <c r="C90" s="6" t="inlineStr">
+        <is>
+          <t>8.25</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>Demo data removed, sections kept</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>All demo shops, products, buyers, orders and reviews deleted from the live site; the 14 home sections kept (empty ones hide)</t>
+        </is>
+      </c>
+      <c r="F90" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G90" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H90" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I90" s="9">
+        <f>IF(AND(G90&lt;&gt;"",H90&lt;&gt;""),H90-G90+1,"")</f>
+        <v/>
+      </c>
+      <c r="J90" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct (seed/demo_remove_keep_sections.sql)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Extra work (added on owner's request)</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="inlineStr">
+        <is>
+          <t>8.26</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>Old demo address forwards</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>rgbkartdemo.hkmanik.com and www.rgbkart.com forward every link to https://rgbkart.com</t>
+        </is>
+      </c>
+      <c r="F91" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G91" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H91" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I91" s="9">
+        <f>IF(AND(G91&lt;&gt;"",H91&lt;&gt;""),H91-G91+1,"")</f>
+        <v/>
+      </c>
+      <c r="J91" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct (.htaccess)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Extra work (added on owner's request)</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr">
+        <is>
+          <t>8.27</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>Live site walk-through checklist</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>Step-by-step list of everything to check on the live site (RGBKart_Live_Site_Checklist.xlsx)</t>
+        </is>
+      </c>
+      <c r="F92" s="7" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="G92" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H92" s="8" t="n"/>
+      <c r="I92" s="9">
+        <f>IF(AND(G92&lt;&gt;"",H92&lt;&gt;""),H92-G92+1,"")</f>
+        <v/>
+      </c>
+      <c r="J92" s="10" t="inlineStr">
+        <is>
+          <t>23 Oct: owner to go through it and note Pass / Fail</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J88"/>
+  <autoFilter ref="A4:J92"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F288">
+  <conditionalFormatting sqref="F5:F292">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$F5="Done"</formula>
     </cfRule>
@@ -4383,10 +4561,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F288" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F292" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Blocked,Done,Not needed"</formula1>
     </dataValidation>
-    <dataValidation sqref="G5:H288" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Enter a date, e.g. 22-Oct-2026" type="date" operator="greaterThan">
+    <dataValidation sqref="G5:H292" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Enter a date, e.g. 22-Oct-2026" type="date" operator="greaterThan">
       <formula1>DATE(2020,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -4485,19 +4663,19 @@
         </is>
       </c>
       <c r="C4" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$288,A4)-COUNTIFS(Plan!$A$5:$A$288,A4,Plan!$F$5:$F$288,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$292,A4)-COUNTIFS(Plan!$A$5:$A$292,A4,Plan!$F$5:$F$292,"Not needed")</f>
         <v/>
       </c>
       <c r="D4" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A4,Plan!$F$5:$F$288,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A4,Plan!$F$5:$F$292,"Done")</f>
         <v/>
       </c>
       <c r="E4" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A4,Plan!$F$5:$F$288,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A4,Plan!$F$5:$F$292,"In progress")</f>
         <v/>
       </c>
       <c r="F4" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A4,Plan!$F$5:$F$288,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A4,Plan!$F$5:$F$292,"Blocked")</f>
         <v/>
       </c>
       <c r="G4" s="15">
@@ -4509,11 +4687,11 @@
         <v/>
       </c>
       <c r="I4" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A4)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A4))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A4)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A4))</f>
         <v/>
       </c>
       <c r="J4" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A4)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A4))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A4)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A4))</f>
         <v/>
       </c>
     </row>
@@ -4527,19 +4705,19 @@
         </is>
       </c>
       <c r="C5" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$288,A5)-COUNTIFS(Plan!$A$5:$A$288,A5,Plan!$F$5:$F$288,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$292,A5)-COUNTIFS(Plan!$A$5:$A$292,A5,Plan!$F$5:$F$292,"Not needed")</f>
         <v/>
       </c>
       <c r="D5" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A5,Plan!$F$5:$F$288,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A5,Plan!$F$5:$F$292,"Done")</f>
         <v/>
       </c>
       <c r="E5" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A5,Plan!$F$5:$F$288,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A5,Plan!$F$5:$F$292,"In progress")</f>
         <v/>
       </c>
       <c r="F5" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A5,Plan!$F$5:$F$288,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A5,Plan!$F$5:$F$292,"Blocked")</f>
         <v/>
       </c>
       <c r="G5" s="15">
@@ -4551,11 +4729,11 @@
         <v/>
       </c>
       <c r="I5" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A5)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A5))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A5)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A5))</f>
         <v/>
       </c>
       <c r="J5" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A5)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A5))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A5)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A5))</f>
         <v/>
       </c>
     </row>
@@ -4569,19 +4747,19 @@
         </is>
       </c>
       <c r="C6" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$288,A6)-COUNTIFS(Plan!$A$5:$A$288,A6,Plan!$F$5:$F$288,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$292,A6)-COUNTIFS(Plan!$A$5:$A$292,A6,Plan!$F$5:$F$292,"Not needed")</f>
         <v/>
       </c>
       <c r="D6" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A6,Plan!$F$5:$F$288,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A6,Plan!$F$5:$F$292,"Done")</f>
         <v/>
       </c>
       <c r="E6" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A6,Plan!$F$5:$F$288,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A6,Plan!$F$5:$F$292,"In progress")</f>
         <v/>
       </c>
       <c r="F6" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A6,Plan!$F$5:$F$288,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A6,Plan!$F$5:$F$292,"Blocked")</f>
         <v/>
       </c>
       <c r="G6" s="15">
@@ -4593,11 +4771,11 @@
         <v/>
       </c>
       <c r="I6" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A6)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A6))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A6)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A6))</f>
         <v/>
       </c>
       <c r="J6" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A6)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A6))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A6)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A6))</f>
         <v/>
       </c>
     </row>
@@ -4611,19 +4789,19 @@
         </is>
       </c>
       <c r="C7" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$288,A7)-COUNTIFS(Plan!$A$5:$A$288,A7,Plan!$F$5:$F$288,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$292,A7)-COUNTIFS(Plan!$A$5:$A$292,A7,Plan!$F$5:$F$292,"Not needed")</f>
         <v/>
       </c>
       <c r="D7" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A7,Plan!$F$5:$F$288,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A7,Plan!$F$5:$F$292,"Done")</f>
         <v/>
       </c>
       <c r="E7" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A7,Plan!$F$5:$F$288,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A7,Plan!$F$5:$F$292,"In progress")</f>
         <v/>
       </c>
       <c r="F7" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A7,Plan!$F$5:$F$288,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A7,Plan!$F$5:$F$292,"Blocked")</f>
         <v/>
       </c>
       <c r="G7" s="15">
@@ -4635,11 +4813,11 @@
         <v/>
       </c>
       <c r="I7" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A7)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A7))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A7)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A7))</f>
         <v/>
       </c>
       <c r="J7" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A7)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A7))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A7)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A7))</f>
         <v/>
       </c>
     </row>
@@ -4653,19 +4831,19 @@
         </is>
       </c>
       <c r="C8" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$288,A8)-COUNTIFS(Plan!$A$5:$A$288,A8,Plan!$F$5:$F$288,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$292,A8)-COUNTIFS(Plan!$A$5:$A$292,A8,Plan!$F$5:$F$292,"Not needed")</f>
         <v/>
       </c>
       <c r="D8" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A8,Plan!$F$5:$F$288,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A8,Plan!$F$5:$F$292,"Done")</f>
         <v/>
       </c>
       <c r="E8" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A8,Plan!$F$5:$F$288,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A8,Plan!$F$5:$F$292,"In progress")</f>
         <v/>
       </c>
       <c r="F8" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A8,Plan!$F$5:$F$288,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A8,Plan!$F$5:$F$292,"Blocked")</f>
         <v/>
       </c>
       <c r="G8" s="15">
@@ -4677,11 +4855,11 @@
         <v/>
       </c>
       <c r="I8" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A8)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A8))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A8)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A8))</f>
         <v/>
       </c>
       <c r="J8" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A8)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A8))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A8)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A8))</f>
         <v/>
       </c>
     </row>
@@ -4695,19 +4873,19 @@
         </is>
       </c>
       <c r="C9" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$288,A9)-COUNTIFS(Plan!$A$5:$A$288,A9,Plan!$F$5:$F$288,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$292,A9)-COUNTIFS(Plan!$A$5:$A$292,A9,Plan!$F$5:$F$292,"Not needed")</f>
         <v/>
       </c>
       <c r="D9" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A9,Plan!$F$5:$F$288,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A9,Plan!$F$5:$F$292,"Done")</f>
         <v/>
       </c>
       <c r="E9" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A9,Plan!$F$5:$F$288,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A9,Plan!$F$5:$F$292,"In progress")</f>
         <v/>
       </c>
       <c r="F9" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A9,Plan!$F$5:$F$288,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A9,Plan!$F$5:$F$292,"Blocked")</f>
         <v/>
       </c>
       <c r="G9" s="15">
@@ -4719,11 +4897,11 @@
         <v/>
       </c>
       <c r="I9" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A9)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A9))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A9)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A9))</f>
         <v/>
       </c>
       <c r="J9" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A9)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A9))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A9)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A9))</f>
         <v/>
       </c>
     </row>
@@ -4737,19 +4915,19 @@
         </is>
       </c>
       <c r="C10" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$288,A10)-COUNTIFS(Plan!$A$5:$A$288,A10,Plan!$F$5:$F$288,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$292,A10)-COUNTIFS(Plan!$A$5:$A$292,A10,Plan!$F$5:$F$292,"Not needed")</f>
         <v/>
       </c>
       <c r="D10" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A10,Plan!$F$5:$F$288,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A10,Plan!$F$5:$F$292,"Done")</f>
         <v/>
       </c>
       <c r="E10" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A10,Plan!$F$5:$F$288,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A10,Plan!$F$5:$F$292,"In progress")</f>
         <v/>
       </c>
       <c r="F10" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A10,Plan!$F$5:$F$288,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A10,Plan!$F$5:$F$292,"Blocked")</f>
         <v/>
       </c>
       <c r="G10" s="15">
@@ -4761,11 +4939,11 @@
         <v/>
       </c>
       <c r="I10" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A10)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A10))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A10)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A10))</f>
         <v/>
       </c>
       <c r="J10" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A10)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A10))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A10)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A10))</f>
         <v/>
       </c>
     </row>
@@ -4779,19 +4957,19 @@
         </is>
       </c>
       <c r="C11" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$288,A11)-COUNTIFS(Plan!$A$5:$A$288,A11,Plan!$F$5:$F$288,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$292,A11)-COUNTIFS(Plan!$A$5:$A$292,A11,Plan!$F$5:$F$292,"Not needed")</f>
         <v/>
       </c>
       <c r="D11" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A11,Plan!$F$5:$F$288,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A11,Plan!$F$5:$F$292,"Done")</f>
         <v/>
       </c>
       <c r="E11" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A11,Plan!$F$5:$F$288,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A11,Plan!$F$5:$F$292,"In progress")</f>
         <v/>
       </c>
       <c r="F11" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A11,Plan!$F$5:$F$288,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A11,Plan!$F$5:$F$292,"Blocked")</f>
         <v/>
       </c>
       <c r="G11" s="15">
@@ -4803,11 +4981,11 @@
         <v/>
       </c>
       <c r="I11" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A11)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A11))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A11)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A11))</f>
         <v/>
       </c>
       <c r="J11" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A11)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A11))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A11)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A11))</f>
         <v/>
       </c>
     </row>
@@ -4821,19 +4999,19 @@
         </is>
       </c>
       <c r="C12" s="15">
-        <f>COUNTIF(Plan!$A$5:$A$288,A12)-COUNTIFS(Plan!$A$5:$A$288,A12,Plan!$F$5:$F$288,"Not needed")</f>
+        <f>COUNTIF(Plan!$A$5:$A$292,A12)-COUNTIFS(Plan!$A$5:$A$292,A12,Plan!$F$5:$F$292,"Not needed")</f>
         <v/>
       </c>
       <c r="D12" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A12,Plan!$F$5:$F$288,"Done")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A12,Plan!$F$5:$F$292,"Done")</f>
         <v/>
       </c>
       <c r="E12" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A12,Plan!$F$5:$F$288,"In progress")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A12,Plan!$F$5:$F$292,"In progress")</f>
         <v/>
       </c>
       <c r="F12" s="15">
-        <f>COUNTIFS(Plan!$A$5:$A$288,$A12,Plan!$F$5:$F$288,"Blocked")</f>
+        <f>COUNTIFS(Plan!$A$5:$A$292,$A12,Plan!$F$5:$F$292,"Blocked")</f>
         <v/>
       </c>
       <c r="G12" s="15">
@@ -4845,11 +5023,11 @@
         <v/>
       </c>
       <c r="I12" s="17">
-        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A12)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$288,Plan!$A$5:$A$288,A12))</f>
+        <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A12)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$292,Plan!$A$5:$A$292,A12))</f>
         <v/>
       </c>
       <c r="J12" s="17">
-        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A12)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$288,Plan!$A$5:$A$288,A12))</f>
+        <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A12)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$292,Plan!$A$5:$A$292,A12))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan 0.4: Google sign-in live; Facebook still to do
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SVU1RwqVH7nME6a6jQM3H6
</commit_message>
<xml_diff>
--- a/docs/RGBKart_Project_Plan.xlsx
+++ b/docs/RGBKart_Project_Plan.xlsx
@@ -19,9 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="dd-mmm-yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd-mmm-yyyy"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -97,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -116,7 +115,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -139,9 +138,13 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -605,6 +608,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -686,10 +690,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G5" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H5" s="8" t="n">
+      <c r="G5" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H5" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I5" s="9">
@@ -731,10 +735,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G6" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H6" s="8" t="n">
+      <c r="G6" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H6" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I6" s="9">
@@ -772,10 +776,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G7" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H7" s="8" t="n">
+      <c r="G7" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H7" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I7" s="9">
@@ -817,17 +821,17 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G8" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H8" s="8" t="n"/>
+      <c r="G8" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H8" s="20" t="n"/>
       <c r="I8" s="9">
         <f>IF(AND(G8&lt;&gt;"",H8&lt;&gt;""),H8-G8+1,"")</f>
         <v/>
       </c>
       <c r="J8" s="10" t="inlineStr">
         <is>
-          <t>Code done. To do: Google Cloud OAuth client, Meta app, enable both in Supabase, set Site URL + Redirect URLs</t>
+          <t>Code done. 24 Oct: Google LIVE (Google Cloud project RGBKart, consent screen in production, web client, enabled in Supabase; tested with a new account). To do: Meta app for Facebook, enable in Supabase.</t>
         </is>
       </c>
     </row>
@@ -860,10 +864,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G9" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H9" s="8" t="n">
+      <c r="G9" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H9" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I9" s="9">
@@ -905,10 +909,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G10" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H10" s="8" t="n">
+      <c r="G10" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H10" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I10" s="9">
@@ -950,10 +954,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G11" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H11" s="8" t="n">
+      <c r="G11" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H11" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I11" s="9">
@@ -995,10 +999,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G12" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H12" s="8" t="n">
+      <c r="G12" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H12" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I12" s="14">
@@ -1040,10 +1044,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G13" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H13" s="8" t="n">
+      <c r="G13" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H13" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I13" s="14">
@@ -1085,10 +1089,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G14" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H14" s="8" t="n">
+      <c r="G14" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H14" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I14" s="14">
@@ -1130,10 +1134,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G15" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H15" s="8" t="n">
+      <c r="G15" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H15" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I15" s="14">
@@ -1175,10 +1179,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G16" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H16" s="8" t="n">
+      <c r="G16" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H16" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I16" s="14">
@@ -1220,10 +1224,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G17" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H17" s="8" t="n">
+      <c r="G17" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H17" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I17" s="14">
@@ -1265,10 +1269,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G18" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H18" s="8" t="n">
+      <c r="G18" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H18" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I18" s="14">
@@ -1310,10 +1314,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G19" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H19" s="8" t="n">
+      <c r="G19" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H19" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I19" s="14">
@@ -1355,10 +1359,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G20" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H20" s="8" t="n"/>
+      <c r="G20" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H20" s="20" t="n"/>
       <c r="I20" s="9">
         <f>IF(AND(G20&lt;&gt;"",H20&lt;&gt;""),H20-G20+1,"")</f>
         <v/>
@@ -1398,10 +1402,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G21" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H21" s="8" t="n"/>
+      <c r="G21" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H21" s="20" t="n"/>
       <c r="I21" s="9">
         <f>IF(AND(G21&lt;&gt;"",H21&lt;&gt;""),H21-G21+1,"")</f>
         <v/>
@@ -1441,10 +1445,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G22" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H22" s="8" t="n">
+      <c r="G22" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H22" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I22" s="9">
@@ -1486,10 +1490,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G23" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H23" s="8" t="n"/>
+      <c r="G23" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H23" s="20" t="n"/>
       <c r="I23" s="9">
         <f>IF(AND(G23&lt;&gt;"",H23&lt;&gt;""),H23-G23+1,"")</f>
         <v/>
@@ -1529,10 +1533,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G24" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H24" s="8" t="n">
+      <c r="G24" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H24" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I24" s="9">
@@ -1574,10 +1578,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G25" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H25" s="8" t="n">
+      <c r="G25" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H25" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I25" s="9">
@@ -1619,10 +1623,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G26" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H26" s="8" t="n">
+      <c r="G26" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H26" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I26" s="9">
@@ -1664,10 +1668,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G27" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H27" s="8" t="n"/>
+      <c r="G27" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H27" s="20" t="n"/>
       <c r="I27" s="9">
         <f>IF(AND(G27&lt;&gt;"",H27&lt;&gt;""),H27-G27+1,"")</f>
         <v/>
@@ -1707,10 +1711,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G28" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H28" s="8" t="n">
+      <c r="G28" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H28" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I28" s="14">
@@ -1752,10 +1756,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G29" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H29" s="8" t="n"/>
+      <c r="G29" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H29" s="20" t="n"/>
       <c r="I29" s="14">
         <f>IF(AND(G29&lt;&gt;"",H29&lt;&gt;""),H29-G29+1,"")</f>
         <v/>
@@ -1795,10 +1799,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G30" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H30" s="8" t="n">
+      <c r="G30" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H30" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I30" s="14">
@@ -1840,8 +1844,8 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="G31" s="8" t="n"/>
-      <c r="H31" s="8" t="n"/>
+      <c r="G31" s="20" t="n"/>
+      <c r="H31" s="20" t="n"/>
       <c r="I31" s="14">
         <f>IF(AND(G31&lt;&gt;"",H31&lt;&gt;""),H31-G31+1,"")</f>
         <v/>
@@ -1881,8 +1885,8 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="G32" s="8" t="n"/>
-      <c r="H32" s="8" t="n"/>
+      <c r="G32" s="20" t="n"/>
+      <c r="H32" s="20" t="n"/>
       <c r="I32" s="14">
         <f>IF(AND(G32&lt;&gt;"",H32&lt;&gt;""),H32-G32+1,"")</f>
         <v/>
@@ -1922,10 +1926,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G33" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H33" s="8" t="n">
+      <c r="G33" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H33" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I33" s="14">
@@ -1967,10 +1971,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G34" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H34" s="8" t="n"/>
+      <c r="G34" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H34" s="20" t="n"/>
       <c r="I34" s="14">
         <f>IF(AND(G34&lt;&gt;"",H34&lt;&gt;""),H34-G34+1,"")</f>
         <v/>
@@ -2010,10 +2014,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G35" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H35" s="8" t="n"/>
+      <c r="G35" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H35" s="20" t="n"/>
       <c r="I35" s="9">
         <f>IF(AND(G35&lt;&gt;"",H35&lt;&gt;""),H35-G35+1,"")</f>
         <v/>
@@ -2053,10 +2057,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G36" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H36" s="8" t="n"/>
+      <c r="G36" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H36" s="20" t="n"/>
       <c r="I36" s="9">
         <f>IF(AND(G36&lt;&gt;"",H36&lt;&gt;""),H36-G36+1,"")</f>
         <v/>
@@ -2096,8 +2100,8 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="G37" s="8" t="n"/>
-      <c r="H37" s="8" t="n"/>
+      <c r="G37" s="20" t="n"/>
+      <c r="H37" s="20" t="n"/>
       <c r="I37" s="9">
         <f>IF(AND(G37&lt;&gt;"",H37&lt;&gt;""),H37-G37+1,"")</f>
         <v/>
@@ -2137,10 +2141,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G38" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H38" s="8" t="n"/>
+      <c r="G38" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H38" s="20" t="n"/>
       <c r="I38" s="9">
         <f>IF(AND(G38&lt;&gt;"",H38&lt;&gt;""),H38-G38+1,"")</f>
         <v/>
@@ -2180,10 +2184,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G39" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H39" s="8" t="n">
+      <c r="G39" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H39" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I39" s="9">
@@ -2225,10 +2229,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G40" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H40" s="8" t="n">
+      <c r="G40" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H40" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I40" s="9">
@@ -2270,8 +2274,8 @@
           <t>Not needed</t>
         </is>
       </c>
-      <c r="G41" s="8" t="n"/>
-      <c r="H41" s="8" t="n"/>
+      <c r="G41" s="20" t="n"/>
+      <c r="H41" s="20" t="n"/>
       <c r="I41" s="14">
         <f>IF(AND(G41&lt;&gt;"",H41&lt;&gt;""),H41-G41+1,"")</f>
         <v/>
@@ -2311,8 +2315,8 @@
           <t>Not needed</t>
         </is>
       </c>
-      <c r="G42" s="8" t="n"/>
-      <c r="H42" s="8" t="n"/>
+      <c r="G42" s="20" t="n"/>
+      <c r="H42" s="20" t="n"/>
       <c r="I42" s="14">
         <f>IF(AND(G42&lt;&gt;"",H42&lt;&gt;""),H42-G42+1,"")</f>
         <v/>
@@ -2352,8 +2356,8 @@
           <t>Not needed</t>
         </is>
       </c>
-      <c r="G43" s="8" t="n"/>
-      <c r="H43" s="8" t="n"/>
+      <c r="G43" s="20" t="n"/>
+      <c r="H43" s="20" t="n"/>
       <c r="I43" s="14">
         <f>IF(AND(G43&lt;&gt;"",H43&lt;&gt;""),H43-G43+1,"")</f>
         <v/>
@@ -2393,10 +2397,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G44" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H44" s="8" t="n"/>
+      <c r="G44" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H44" s="20" t="n"/>
       <c r="I44" s="14">
         <f>IF(AND(G44&lt;&gt;"",H44&lt;&gt;""),H44-G44+1,"")</f>
         <v/>
@@ -2436,10 +2440,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G45" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H45" s="8" t="n"/>
+      <c r="G45" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H45" s="20" t="n"/>
       <c r="I45" s="14">
         <f>IF(AND(G45&lt;&gt;"",H45&lt;&gt;""),H45-G45+1,"")</f>
         <v/>
@@ -2479,10 +2483,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G46" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H46" s="8" t="n"/>
+      <c r="G46" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H46" s="20" t="n"/>
       <c r="I46" s="14">
         <f>IF(AND(G46&lt;&gt;"",H46&lt;&gt;""),H46-G46+1,"")</f>
         <v/>
@@ -2522,10 +2526,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G47" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H47" s="8" t="n"/>
+      <c r="G47" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H47" s="20" t="n"/>
       <c r="I47" s="14">
         <f>IF(AND(G47&lt;&gt;"",H47&lt;&gt;""),H47-G47+1,"")</f>
         <v/>
@@ -2565,10 +2569,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G48" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H48" s="8" t="n"/>
+      <c r="G48" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H48" s="20" t="n"/>
       <c r="I48" s="14">
         <f>IF(AND(G48&lt;&gt;"",H48&lt;&gt;""),H48-G48+1,"")</f>
         <v/>
@@ -2608,10 +2612,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G49" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H49" s="8" t="n"/>
+      <c r="G49" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H49" s="20" t="n"/>
       <c r="I49" s="14">
         <f>IF(AND(G49&lt;&gt;"",H49&lt;&gt;""),H49-G49+1,"")</f>
         <v/>
@@ -2651,10 +2655,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G50" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H50" s="8" t="n">
+      <c r="G50" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H50" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I50" s="14">
@@ -2696,10 +2700,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G51" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H51" s="8" t="n">
+      <c r="G51" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H51" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I51" s="14">
@@ -2741,10 +2745,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G52" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H52" s="8" t="n">
+      <c r="G52" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H52" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I52" s="9">
@@ -2786,10 +2790,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G53" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H53" s="8" t="n">
+      <c r="G53" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H53" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I53" s="9">
@@ -2831,10 +2835,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G54" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H54" s="8" t="n">
+      <c r="G54" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H54" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I54" s="9">
@@ -2876,10 +2880,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G55" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H55" s="8" t="n">
+      <c r="G55" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H55" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I55" s="9">
@@ -2921,10 +2925,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G56" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H56" s="8" t="n">
+      <c r="G56" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H56" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I56" s="9">
@@ -2966,10 +2970,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G57" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H57" s="8" t="n">
+      <c r="G57" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H57" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I57" s="14">
@@ -3011,10 +3015,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G58" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H58" s="8" t="n">
+      <c r="G58" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H58" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I58" s="14">
@@ -3056,10 +3060,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G59" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H59" s="8" t="n"/>
+      <c r="G59" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H59" s="20" t="n"/>
       <c r="I59" s="14">
         <f>IF(AND(G59&lt;&gt;"",H59&lt;&gt;""),H59-G59+1,"")</f>
         <v/>
@@ -3099,10 +3103,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G60" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H60" s="8" t="n"/>
+      <c r="G60" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H60" s="20" t="n"/>
       <c r="I60" s="14">
         <f>IF(AND(G60&lt;&gt;"",H60&lt;&gt;""),H60-G60+1,"")</f>
         <v/>
@@ -3142,10 +3146,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G61" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H61" s="8" t="n"/>
+      <c r="G61" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H61" s="20" t="n"/>
       <c r="I61" s="14">
         <f>IF(AND(G61&lt;&gt;"",H61&lt;&gt;""),H61-G61+1,"")</f>
         <v/>
@@ -3185,10 +3189,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G62" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H62" s="8" t="n">
+      <c r="G62" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H62" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I62" s="14">
@@ -3230,8 +3234,8 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="G63" s="8" t="n"/>
-      <c r="H63" s="8" t="n"/>
+      <c r="G63" s="20" t="n"/>
+      <c r="H63" s="20" t="n"/>
       <c r="I63" s="14">
         <f>IF(AND(G63&lt;&gt;"",H63&lt;&gt;""),H63-G63+1,"")</f>
         <v/>
@@ -3267,10 +3271,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G64" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H64" s="8" t="n">
+      <c r="G64" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H64" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I64" s="14">
@@ -3312,10 +3316,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G65" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H65" s="8" t="n">
+      <c r="G65" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H65" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I65" s="14">
@@ -3357,10 +3361,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G66" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H66" s="8" t="n">
+      <c r="G66" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H66" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I66" s="9">
@@ -3402,10 +3406,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G67" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H67" s="8" t="n">
+      <c r="G67" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H67" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I67" s="9">
@@ -3447,10 +3451,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G68" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H68" s="8" t="n">
+      <c r="G68" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H68" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I68" s="9">
@@ -3492,10 +3496,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G69" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H69" s="8" t="n">
+      <c r="G69" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H69" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I69" s="9">
@@ -3537,10 +3541,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G70" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H70" s="8" t="n">
+      <c r="G70" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H70" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I70" s="9">
@@ -3582,10 +3586,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G71" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H71" s="8" t="n">
+      <c r="G71" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H71" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="I71" s="9">
@@ -3627,10 +3631,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G72" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H72" s="8" t="n">
+      <c r="G72" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H72" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I72" s="9">
@@ -3672,10 +3676,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G73" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H73" s="8" t="n">
+      <c r="G73" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H73" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I73" s="9">
@@ -3717,10 +3721,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G74" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H74" s="8" t="n">
+      <c r="G74" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H74" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I74" s="9">
@@ -3762,10 +3766,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G75" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H75" s="8" t="n">
+      <c r="G75" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H75" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I75" s="9">
@@ -3807,10 +3811,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G76" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H76" s="8" t="n">
+      <c r="G76" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H76" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I76" s="9">
@@ -3852,10 +3856,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G77" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H77" s="8" t="n">
+      <c r="G77" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H77" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I77" s="9">
@@ -3897,10 +3901,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G78" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H78" s="8" t="n">
+      <c r="G78" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H78" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I78" s="9">
@@ -3942,10 +3946,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G79" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H79" s="8" t="n">
+      <c r="G79" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H79" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I79" s="9">
@@ -3987,10 +3991,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G80" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H80" s="8" t="n">
+      <c r="G80" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H80" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I80" s="9">
@@ -4032,10 +4036,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G81" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H81" s="8" t="n">
+      <c r="G81" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H81" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I81" s="9">
@@ -4077,10 +4081,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G82" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H82" s="8" t="n">
+      <c r="G82" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H82" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I82" s="9">
@@ -4122,10 +4126,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G83" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H83" s="8" t="n">
+      <c r="G83" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H83" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I83" s="9">
@@ -4167,10 +4171,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G84" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H84" s="8" t="n">
+      <c r="G84" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H84" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I84" s="9">
@@ -4212,10 +4216,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G85" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H85" s="8" t="n">
+      <c r="G85" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H85" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I85" s="9">
@@ -4257,10 +4261,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G86" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H86" s="8" t="n">
+      <c r="G86" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H86" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I86" s="9">
@@ -4302,10 +4306,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G87" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H87" s="8" t="n">
+      <c r="G87" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H87" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I87" s="9">
@@ -4347,10 +4351,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G88" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H88" s="8" t="n">
+      <c r="G88" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H88" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I88" s="9">
@@ -4392,10 +4396,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G89" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H89" s="8" t="n">
+      <c r="G89" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H89" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I89" s="9">
@@ -4437,10 +4441,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G90" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H90" s="8" t="n">
+      <c r="G90" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H90" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I90" s="9">
@@ -4482,10 +4486,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G91" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H91" s="8" t="n">
+      <c r="G91" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H91" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I91" s="9">
@@ -4527,10 +4531,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="G92" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H92" s="8" t="n">
+      <c r="G92" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H92" s="20" t="n">
         <v>46318</v>
       </c>
       <c r="I92" s="9">
@@ -4572,10 +4576,10 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="G93" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H93" s="8" t="n"/>
+      <c r="G93" s="20" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H93" s="20" t="n"/>
       <c r="I93" s="9">
         <f>IF(AND(G93&lt;&gt;"",H93&lt;&gt;""),H93-G93+1,"")</f>
         <v/>
@@ -4646,6 +4650,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -4731,11 +4736,11 @@
         <f>IF(C4=0,0,D4/C4)</f>
         <v/>
       </c>
-      <c r="I4" s="17">
+      <c r="I4" s="21">
         <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A4)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A4))</f>
         <v/>
       </c>
-      <c r="J4" s="17">
+      <c r="J4" s="21">
         <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A4)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A4))</f>
         <v/>
       </c>
@@ -4773,11 +4778,11 @@
         <f>IF(C5=0,0,D5/C5)</f>
         <v/>
       </c>
-      <c r="I5" s="17">
+      <c r="I5" s="21">
         <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A5)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A5))</f>
         <v/>
       </c>
-      <c r="J5" s="17">
+      <c r="J5" s="21">
         <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A5)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A5))</f>
         <v/>
       </c>
@@ -4815,11 +4820,11 @@
         <f>IF(C6=0,0,D6/C6)</f>
         <v/>
       </c>
-      <c r="I6" s="17">
+      <c r="I6" s="21">
         <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A6)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A6))</f>
         <v/>
       </c>
-      <c r="J6" s="17">
+      <c r="J6" s="21">
         <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A6)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A6))</f>
         <v/>
       </c>
@@ -4857,11 +4862,11 @@
         <f>IF(C7=0,0,D7/C7)</f>
         <v/>
       </c>
-      <c r="I7" s="17">
+      <c r="I7" s="21">
         <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A7)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A7))</f>
         <v/>
       </c>
-      <c r="J7" s="17">
+      <c r="J7" s="21">
         <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A7)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A7))</f>
         <v/>
       </c>
@@ -4899,11 +4904,11 @@
         <f>IF(C8=0,0,D8/C8)</f>
         <v/>
       </c>
-      <c r="I8" s="17">
+      <c r="I8" s="21">
         <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A8)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A8))</f>
         <v/>
       </c>
-      <c r="J8" s="17">
+      <c r="J8" s="21">
         <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A8)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A8))</f>
         <v/>
       </c>
@@ -4941,11 +4946,11 @@
         <f>IF(C9=0,0,D9/C9)</f>
         <v/>
       </c>
-      <c r="I9" s="17">
+      <c r="I9" s="21">
         <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A9)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A9))</f>
         <v/>
       </c>
-      <c r="J9" s="17">
+      <c r="J9" s="21">
         <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A9)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A9))</f>
         <v/>
       </c>
@@ -4983,11 +4988,11 @@
         <f>IF(C10=0,0,D10/C10)</f>
         <v/>
       </c>
-      <c r="I10" s="17">
+      <c r="I10" s="21">
         <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A10)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A10))</f>
         <v/>
       </c>
-      <c r="J10" s="17">
+      <c r="J10" s="21">
         <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A10)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A10))</f>
         <v/>
       </c>
@@ -5025,11 +5030,11 @@
         <f>IF(C11=0,0,D11/C11)</f>
         <v/>
       </c>
-      <c r="I11" s="17">
+      <c r="I11" s="21">
         <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A11)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A11))</f>
         <v/>
       </c>
-      <c r="J11" s="17">
+      <c r="J11" s="21">
         <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A11)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A11))</f>
         <v/>
       </c>
@@ -5067,11 +5072,11 @@
         <f>IF(C12=0,0,D12/C12)</f>
         <v/>
       </c>
-      <c r="I12" s="17">
+      <c r="I12" s="21">
         <f>IF(_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A12)=0,"",_xlfn.MINIFS(Plan!$G$5:$G$293,Plan!$A$5:$A$293,A12))</f>
         <v/>
       </c>
-      <c r="J12" s="17">
+      <c r="J12" s="21">
         <f>IF(_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A12)=0,"",_xlfn.MAXIFS(Plan!$H$5:$H$293,Plan!$A$5:$A$293,A12))</f>
         <v/>
       </c>
@@ -5110,6 +5115,7 @@
       <c r="I13" s="18" t="n"/>
       <c r="J13" s="18" t="n"/>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>

</xml_diff>